<commit_message>
Update roster 09/2026 from web (24 NV)
</commit_message>
<xml_diff>
--- a/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
+++ b/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN36"/>
+  <dimension ref="A1:AN35"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1407,7 +1407,7 @@
         <v/>
       </c>
       <c r="C18" t="str">
-        <v>Phan Như Ngọc</v>
+        <v>Phan Hiền Phúc Đạt</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -1529,7 +1529,7 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <v>Phan Hiền Phúc Đạt</v>
+        <v>Nguyễn Phạm Quỳnh Trang</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="C20" t="str">
-        <v>Nguyễn Phạm Quỳnh Trang</v>
+        <v>Nguyễn Phương Linh</v>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -1767,19 +1767,19 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v/>
+        <v>DSP HDQ</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>30904</v>
       </c>
       <c r="C21" t="str">
-        <v>Nguyễn Phương Linh</v>
+        <v>Trần Đình Đạt</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -1791,31 +1791,31 @@
         <v/>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K21" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="L21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O21" t="str">
         <v/>
       </c>
       <c r="P21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R21" t="str">
         <v/>
@@ -1824,22 +1824,22 @@
         <v/>
       </c>
       <c r="T21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V21" t="str">
         <v/>
       </c>
       <c r="W21" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="X21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z21" t="str">
         <v/>
@@ -1848,10 +1848,10 @@
         <v/>
       </c>
       <c r="AB21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD21" t="str">
         <v/>
@@ -1860,48 +1860,48 @@
         <v/>
       </c>
       <c r="AF21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH21" t="str">
         <v/>
       </c>
       <c r="AI21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ21">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AK21">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AL21">
         <v>0</v>
       </c>
       <c r="AM21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN21">
-        <v>0</v>
+        <v>220</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>DSP HDQ</v>
+        <v/>
       </c>
       <c r="B22" t="str">
-        <v>30904</v>
+        <v>30905</v>
       </c>
       <c r="C22" t="str">
-        <v>Trần Đình Đạt</v>
+        <v>Nguyễn Trương Hoàng Hưng</v>
       </c>
       <c r="D22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="E22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -1910,94 +1910,94 @@
         <v/>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="J22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="K22" t="str">
         <v>NL</v>
       </c>
       <c r="L22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="N22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O22" t="str">
         <v/>
       </c>
       <c r="P22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V22" t="str">
         <v/>
       </c>
       <c r="W22" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="X22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE22" t="str">
         <v/>
       </c>
       <c r="AF22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AH22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AI22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ22">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AK22">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AL22">
         <v>0</v>
@@ -2006,7 +2006,7 @@
         <v>1</v>
       </c>
       <c r="AN22">
-        <v>220</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23">
@@ -2014,46 +2014,46 @@
         <v/>
       </c>
       <c r="B23" t="str">
-        <v>30905</v>
+        <v>30841</v>
       </c>
       <c r="C23" t="str">
-        <v>Nguyễn Trương Hoàng Hưng</v>
+        <v>Vũ Hoàng Long</v>
       </c>
       <c r="D23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="H23" t="str">
-        <v>M</v>
+        <v>P</v>
       </c>
       <c r="I23" t="str">
-        <v>E</v>
+        <v>P</v>
       </c>
       <c r="J23" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="K23" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L23" t="str">
         <v/>
       </c>
       <c r="M23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P23" t="str">
         <v>E</v>
@@ -2065,22 +2065,22 @@
         <v>M</v>
       </c>
       <c r="S23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U23" t="str">
         <v/>
       </c>
       <c r="V23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y23" t="str">
         <v/>
@@ -2089,37 +2089,37 @@
         <v>M</v>
       </c>
       <c r="AA23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AB23" t="str">
         <v/>
       </c>
       <c r="AC23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AH23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AI23">
         <v>0</v>
       </c>
       <c r="AJ23">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK23">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AL23">
         <v>0</v>
@@ -2128,7 +2128,7 @@
         <v>1</v>
       </c>
       <c r="AN23">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="24">
@@ -2136,97 +2136,97 @@
         <v/>
       </c>
       <c r="B24" t="str">
-        <v>30841</v>
+        <v>29718</v>
       </c>
       <c r="C24" t="str">
-        <v>Vũ Hoàng Long</v>
+        <v>Vũ Huy Hùng</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="E24" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="F24" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="G24" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="H24" t="str">
-        <v>P</v>
+        <v/>
       </c>
       <c r="I24" t="str">
-        <v>P</v>
+        <v>HC</v>
       </c>
       <c r="J24" t="str">
+        <v>M</v>
+      </c>
+      <c r="K24" t="str">
         <v>NL</v>
       </c>
-      <c r="K24" t="str">
-        <v>E</v>
-      </c>
       <c r="L24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="O24" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="P24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T24" t="str">
         <v/>
       </c>
       <c r="U24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X24" t="str">
         <v/>
       </c>
       <c r="Y24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AG24" t="str">
         <v/>
@@ -2235,10 +2235,10 @@
         <v>M</v>
       </c>
       <c r="AI24">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ24">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AK24">
         <v>7</v>
@@ -2255,49 +2255,49 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v>DSP ASST HDQ</v>
       </c>
       <c r="B25" t="str">
-        <v>29718</v>
+        <v>39278</v>
       </c>
       <c r="C25" t="str">
-        <v>Vũ Huy Hùng</v>
+        <v>Nguyền Kiều Huyền Chi</v>
       </c>
       <c r="D25" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="E25" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="F25" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="G25" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="H25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I25" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="J25" t="str">
         <v>M</v>
       </c>
       <c r="K25" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="L25" t="str">
         <v>E</v>
       </c>
       <c r="M25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N25" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="O25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P25" t="str">
         <v/>
@@ -2306,10 +2306,10 @@
         <v>M</v>
       </c>
       <c r="R25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="S25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T25" t="str">
         <v/>
@@ -2321,165 +2321,165 @@
         <v>E</v>
       </c>
       <c r="W25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X25" t="str">
         <v/>
       </c>
       <c r="Y25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Z25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AA25" t="str">
         <v/>
       </c>
       <c r="AB25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC25" t="str">
         <v/>
       </c>
       <c r="AD25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AE25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF25" t="str">
-        <v/>
+        <v>C349</v>
       </c>
       <c r="AG25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AH25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AI25">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ25">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AK25">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AL25">
         <v>0</v>
       </c>
       <c r="AM25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN25">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>DSP ASST HDQ</v>
+        <v/>
       </c>
       <c r="B26" t="str">
-        <v>39278</v>
+        <v>39280</v>
       </c>
       <c r="C26" t="str">
-        <v>Nguyền Kiều Huyền Chi</v>
+        <v>Đặng Thảo Linh</v>
       </c>
       <c r="D26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E26" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="H26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="I26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J26" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="K26" t="str">
         <v>M</v>
       </c>
       <c r="L26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="M26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N26" t="str">
-        <v>SN</v>
+        <v/>
       </c>
       <c r="O26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="P26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="R26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T26" t="str">
         <v/>
       </c>
       <c r="U26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="X26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y26" t="str">
         <v/>
       </c>
       <c r="Z26" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="AA26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE26" t="str">
         <v/>
       </c>
       <c r="AF26" t="str">
-        <v>C349</v>
+        <v>M</v>
       </c>
       <c r="AG26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AH26" t="str">
         <v>E</v>
       </c>
       <c r="AI26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ26">
         <v>8</v>
@@ -2491,10 +2491,10 @@
         <v>0</v>
       </c>
       <c r="AM26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN26">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27">
@@ -2502,64 +2502,64 @@
         <v/>
       </c>
       <c r="B27" t="str">
-        <v>39280</v>
+        <v>39276</v>
       </c>
       <c r="C27" t="str">
-        <v>Đặng Thảo Linh</v>
+        <v>Bùi Việt Anh</v>
       </c>
       <c r="D27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I27" t="str">
         <v>E</v>
       </c>
       <c r="J27" t="str">
+        <v>E</v>
+      </c>
+      <c r="K27" t="str">
         <v>NL</v>
       </c>
-      <c r="K27" t="str">
-        <v>M</v>
-      </c>
       <c r="L27" t="str">
-        <v>M</v>
+        <v>P</v>
       </c>
       <c r="M27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="P27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V27" t="str">
         <v/>
@@ -2568,46 +2568,46 @@
         <v>M</v>
       </c>
       <c r="X27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z27" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AA27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AB27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH27" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AI27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ27">
+        <v>9</v>
+      </c>
+      <c r="AK27">
         <v>8</v>
-      </c>
-      <c r="AK27">
-        <v>9</v>
       </c>
       <c r="AL27">
         <v>0</v>
@@ -2624,19 +2624,19 @@
         <v/>
       </c>
       <c r="B28" t="str">
-        <v>39276</v>
+        <v>39274</v>
       </c>
       <c r="C28" t="str">
-        <v>Bùi Việt Anh</v>
+        <v>Đỗ Nam Anh</v>
       </c>
       <c r="D28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="E28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G28" t="str">
         <v/>
@@ -2645,82 +2645,82 @@
         <v>M</v>
       </c>
       <c r="I28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="J28" t="str">
         <v>E</v>
       </c>
       <c r="K28" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L28" t="str">
-        <v>P</v>
+        <v/>
       </c>
       <c r="M28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O28" t="str">
         <v/>
       </c>
       <c r="P28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R28" t="str">
         <v/>
       </c>
       <c r="S28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="T28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Z28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AA28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AF28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG28" t="str">
         <v/>
       </c>
       <c r="AH28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AI28">
         <v>0</v>
@@ -2729,87 +2729,87 @@
         <v>9</v>
       </c>
       <c r="AK28">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AL28">
         <v>0</v>
       </c>
       <c r="AM28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN28">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v/>
+        <v>DSP SGN</v>
       </c>
       <c r="B29" t="str">
-        <v>39274</v>
+        <v>31844</v>
       </c>
       <c r="C29" t="str">
-        <v>Đỗ Nam Anh</v>
+        <v>Nguyễn Hoàng Huy</v>
       </c>
       <c r="D29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="F29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="G29" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="H29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="J29" t="str">
         <v>E</v>
       </c>
       <c r="K29" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="L29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M29" t="str">
         <v>M</v>
       </c>
       <c r="N29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O29" t="str">
         <v/>
       </c>
       <c r="P29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S29" t="str">
         <v/>
       </c>
       <c r="T29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="U29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X29" t="str">
         <v/>
@@ -2818,22 +2818,22 @@
         <v>M</v>
       </c>
       <c r="Z29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA29" t="str">
         <v/>
       </c>
       <c r="AB29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AC29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE29" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="AF29" t="str">
         <v>E</v>
@@ -2842,22 +2842,22 @@
         <v/>
       </c>
       <c r="AH29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AI29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AK29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AL29">
         <v>0</v>
       </c>
       <c r="AM29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN29">
         <v>216</v>
@@ -2865,106 +2865,106 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>DSP SGN</v>
+        <v/>
       </c>
       <c r="B30" t="str">
-        <v>31844</v>
+        <v>31843</v>
       </c>
       <c r="C30" t="str">
-        <v>Nguyễn Hoàng Huy</v>
+        <v>Lương Trung Hiếu</v>
       </c>
       <c r="D30" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G30" t="str">
-        <v>SN</v>
+        <v>E</v>
       </c>
       <c r="H30" t="str">
         <v/>
       </c>
       <c r="I30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J30" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="K30" t="str">
         <v>NL</v>
       </c>
       <c r="L30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O30" t="str">
         <v/>
       </c>
       <c r="P30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="X30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z30" t="str">
         <v/>
       </c>
       <c r="AA30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE30" t="str">
+        <v>M</v>
+      </c>
+      <c r="AF30" t="str">
         <v>HC</v>
       </c>
-      <c r="AF30" t="str">
-        <v>E</v>
-      </c>
       <c r="AG30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AI30">
         <v>1</v>
@@ -2979,7 +2979,7 @@
         <v>0</v>
       </c>
       <c r="AM30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN30">
         <v>216</v>
@@ -2990,61 +2990,61 @@
         <v/>
       </c>
       <c r="B31" t="str">
-        <v>31843</v>
+        <v>31846</v>
       </c>
       <c r="C31" t="str">
-        <v>Lương Trung Hiếu</v>
+        <v>Nguyễn Phúc Thịnh</v>
       </c>
       <c r="D31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="E31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F31" t="str">
         <v/>
       </c>
       <c r="G31" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I31" t="str">
         <v/>
       </c>
       <c r="J31" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="K31" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L31" t="str">
         <v/>
       </c>
       <c r="M31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N31" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="O31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S31" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="T31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U31" t="str">
         <v/>
@@ -3053,19 +3053,19 @@
         <v/>
       </c>
       <c r="W31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="X31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AB31" t="str">
         <v/>
@@ -3074,37 +3074,37 @@
         <v>E</v>
       </c>
       <c r="AD31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AF31" t="str">
+        <v>M</v>
+      </c>
+      <c r="AG31" t="str">
         <v>HC</v>
       </c>
-      <c r="AG31" t="str">
-        <v>E</v>
-      </c>
       <c r="AH31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AI31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK31">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AL31">
         <v>0</v>
       </c>
       <c r="AM31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN31">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32">
@@ -3112,153 +3112,153 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>31846</v>
+        <v>31847</v>
       </c>
       <c r="C32" t="str">
-        <v>Nguyễn Phúc Thịnh</v>
+        <v>Hoàng Bảo Ngọc</v>
       </c>
       <c r="D32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="H32" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="I32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J32" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="K32" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="L32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M32" t="str">
         <v/>
       </c>
       <c r="N32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q32" t="str">
         <v/>
       </c>
       <c r="R32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="S32" t="str">
+        <v>E</v>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
+        <v>M</v>
+      </c>
+      <c r="V32" t="str">
+        <v>M</v>
+      </c>
+      <c r="W32" t="str">
+        <v>E</v>
+      </c>
+      <c r="X32" t="str">
+        <v/>
+      </c>
+      <c r="Y32" t="str">
+        <v/>
+      </c>
+      <c r="Z32" t="str">
+        <v>E</v>
+      </c>
+      <c r="AA32" t="str">
+        <v/>
+      </c>
+      <c r="AB32" t="str">
+        <v>M</v>
+      </c>
+      <c r="AC32" t="str">
+        <v>M</v>
+      </c>
+      <c r="AD32" t="str">
         <v>HC</v>
       </c>
-      <c r="T32" t="str">
-        <v/>
-      </c>
-      <c r="U32" t="str">
-        <v/>
-      </c>
-      <c r="V32" t="str">
-        <v/>
-      </c>
-      <c r="W32" t="str">
-        <v/>
-      </c>
-      <c r="X32" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y32" t="str">
-        <v/>
-      </c>
-      <c r="Z32" t="str">
-        <v>M</v>
-      </c>
-      <c r="AA32" t="str">
-        <v>E</v>
-      </c>
-      <c r="AB32" t="str">
-        <v/>
-      </c>
-      <c r="AC32" t="str">
-        <v>E</v>
-      </c>
-      <c r="AD32" t="str">
-        <v>E</v>
-      </c>
       <c r="AE32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG32" t="str">
+        <v>M</v>
+      </c>
+      <c r="AH32" t="str">
         <v>HC</v>
-      </c>
-      <c r="AH32" t="str">
-        <v>E</v>
       </c>
       <c r="AI32">
         <v>2</v>
       </c>
       <c r="AJ32">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AK32">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AL32">
         <v>0</v>
       </c>
       <c r="AM32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN32">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v/>
+        <v>DSP PQC</v>
       </c>
       <c r="B33" t="str">
-        <v>31847</v>
+        <v>41863</v>
       </c>
       <c r="C33" t="str">
-        <v>Hoàng Bảo Ngọc</v>
+        <v>Lê Ngọc Thành Tài</v>
       </c>
       <c r="D33" t="str">
         <v/>
       </c>
       <c r="E33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F33" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="G33" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="H33" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I33" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="J33" t="str">
-        <v>NL</v>
+        <v>C9</v>
       </c>
       <c r="K33" t="str">
         <v>M</v>
@@ -3270,40 +3270,40 @@
         <v/>
       </c>
       <c r="N33" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="O33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q33" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="R33" t="str">
         <v/>
       </c>
       <c r="S33" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="T33" t="str">
         <v/>
       </c>
       <c r="U33" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V33" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="W33" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y33" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Z33" t="str">
         <v>E</v>
@@ -3312,13 +3312,13 @@
         <v/>
       </c>
       <c r="AB33" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="AC33" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD33" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AE33" t="str">
         <v>E</v>
@@ -3327,25 +3327,25 @@
         <v/>
       </c>
       <c r="AG33" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="AH33" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AI33">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ33">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AK33">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AL33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AM33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN33">
         <v>216</v>
@@ -3353,103 +3353,103 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>DSP PQC</v>
+        <v/>
       </c>
       <c r="B34" t="str">
-        <v>41863</v>
+        <v>41865</v>
       </c>
       <c r="C34" t="str">
-        <v>Lê Ngọc Thành Tài</v>
+        <v>Nguyễn Đức Lộc</v>
       </c>
       <c r="D34" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="E34" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
         <v>C9</v>
       </c>
-      <c r="G34" t="str">
-        <v>E</v>
-      </c>
       <c r="H34" t="str">
         <v/>
       </c>
       <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v>M</v>
+      </c>
+      <c r="K34" t="str">
         <v>C9</v>
       </c>
-      <c r="J34" t="str">
+      <c r="L34" t="str">
         <v>C9</v>
       </c>
-      <c r="K34" t="str">
-        <v>M</v>
-      </c>
-      <c r="L34" t="str">
-        <v>E</v>
-      </c>
       <c r="M34" t="str">
         <v/>
       </c>
       <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
         <v>C9</v>
       </c>
-      <c r="O34" t="str">
-        <v/>
-      </c>
       <c r="P34" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q34" t="str">
+        <v>M</v>
+      </c>
+      <c r="R34" t="str">
         <v>C9</v>
       </c>
-      <c r="R34" t="str">
-        <v/>
-      </c>
       <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
         <v>C9</v>
       </c>
-      <c r="T34" t="str">
-        <v/>
-      </c>
       <c r="U34" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
         <v>C9</v>
       </c>
-      <c r="W34" t="str">
-        <v/>
-      </c>
       <c r="X34" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
+        <v>M</v>
+      </c>
+      <c r="AA34" t="str">
+        <v/>
+      </c>
+      <c r="AB34" t="str">
+        <v/>
+      </c>
+      <c r="AC34" t="str">
         <v>C9</v>
       </c>
-      <c r="Z34" t="str">
-        <v>E</v>
-      </c>
-      <c r="AA34" t="str">
-        <v/>
-      </c>
-      <c r="AB34" t="str">
+      <c r="AD34" t="str">
+        <v/>
+      </c>
+      <c r="AE34" t="str">
         <v>C9</v>
       </c>
-      <c r="AC34" t="str">
-        <v/>
-      </c>
-      <c r="AD34" t="str">
-        <v/>
-      </c>
-      <c r="AE34" t="str">
-        <v>E</v>
-      </c>
       <c r="AF34" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AG34" t="str">
-        <v>C9</v>
+        <v>M</v>
       </c>
       <c r="AH34" t="str">
         <v/>
@@ -3461,10 +3461,10 @@
         <v>4</v>
       </c>
       <c r="AK34">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AL34">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AM34">
         <v>0</v>
@@ -3478,248 +3478,126 @@
         <v/>
       </c>
       <c r="B35" t="str">
-        <v>41865</v>
+        <v>41867</v>
       </c>
       <c r="C35" t="str">
-        <v>Nguyễn Đức Lộc</v>
+        <v>Phan Thành Nghĩa</v>
       </c>
       <c r="D35" t="str">
+        <v>M</v>
+      </c>
+      <c r="E35" t="str">
         <v>C9</v>
       </c>
-      <c r="E35" t="str">
-        <v>E</v>
-      </c>
       <c r="F35" t="str">
         <v/>
       </c>
       <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
         <v>C9</v>
       </c>
-      <c r="H35" t="str">
-        <v/>
-      </c>
       <c r="I35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J35" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="K35" t="str">
+        <v>E</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
         <v>C9</v>
       </c>
-      <c r="L35" t="str">
+      <c r="N35" t="str">
+        <v>E</v>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+      <c r="P35" t="str">
         <v>C9</v>
       </c>
-      <c r="M35" t="str">
-        <v/>
-      </c>
-      <c r="N35" t="str">
-        <v/>
-      </c>
-      <c r="O35" t="str">
+      <c r="Q35" t="str">
+        <v/>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
         <v>C9</v>
       </c>
-      <c r="P35" t="str">
-        <v/>
-      </c>
-      <c r="Q35" t="str">
-        <v>M</v>
-      </c>
-      <c r="R35" t="str">
+      <c r="V35" t="str">
+        <v/>
+      </c>
+      <c r="W35" t="str">
+        <v>M</v>
+      </c>
+      <c r="X35" t="str">
         <v>C9</v>
       </c>
-      <c r="S35" t="str">
-        <v/>
-      </c>
-      <c r="T35" t="str">
+      <c r="Y35" t="str">
+        <v/>
+      </c>
+      <c r="Z35" t="str">
         <v>C9</v>
       </c>
-      <c r="U35" t="str">
-        <v>E</v>
-      </c>
-      <c r="V35" t="str">
-        <v/>
-      </c>
-      <c r="W35" t="str">
+      <c r="AA35" t="str">
         <v>C9</v>
       </c>
-      <c r="X35" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y35" t="str">
-        <v/>
-      </c>
-      <c r="Z35" t="str">
-        <v>M</v>
-      </c>
-      <c r="AA35" t="str">
-        <v/>
-      </c>
       <c r="AB35" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC35" t="str">
+        <v/>
+      </c>
+      <c r="AD35" t="str">
         <v>C9</v>
       </c>
-      <c r="AD35" t="str">
-        <v/>
-      </c>
       <c r="AE35" t="str">
+        <v/>
+      </c>
+      <c r="AF35" t="str">
+        <v/>
+      </c>
+      <c r="AG35" t="str">
+        <v>E</v>
+      </c>
+      <c r="AH35" t="str">
         <v>C9</v>
       </c>
-      <c r="AF35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AG35" t="str">
-        <v>M</v>
-      </c>
-      <c r="AH35" t="str">
-        <v/>
-      </c>
       <c r="AI35">
         <v>0</v>
       </c>
       <c r="AJ35">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AK35">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AL35">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AM35">
         <v>0</v>
       </c>
       <c r="AN35">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v/>
-      </c>
-      <c r="B36" t="str">
-        <v>41867</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Phan Thành Nghĩa</v>
-      </c>
-      <c r="D36" t="str">
-        <v>M</v>
-      </c>
-      <c r="E36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="F36" t="str">
-        <v/>
-      </c>
-      <c r="G36" t="str">
-        <v/>
-      </c>
-      <c r="H36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="I36" t="str">
-        <v>E</v>
-      </c>
-      <c r="J36" t="str">
-        <v>E</v>
-      </c>
-      <c r="K36" t="str">
-        <v>E</v>
-      </c>
-      <c r="L36" t="str">
-        <v/>
-      </c>
-      <c r="M36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="N36" t="str">
-        <v>E</v>
-      </c>
-      <c r="O36" t="str">
-        <v/>
-      </c>
-      <c r="P36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="Q36" t="str">
-        <v/>
-      </c>
-      <c r="R36" t="str">
-        <v/>
-      </c>
-      <c r="S36" t="str">
-        <v/>
-      </c>
-      <c r="T36" t="str">
-        <v/>
-      </c>
-      <c r="U36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="V36" t="str">
-        <v/>
-      </c>
-      <c r="W36" t="str">
-        <v>M</v>
-      </c>
-      <c r="X36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="Y36" t="str">
-        <v/>
-      </c>
-      <c r="Z36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AA36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AB36" t="str">
-        <v>E</v>
-      </c>
-      <c r="AC36" t="str">
-        <v/>
-      </c>
-      <c r="AD36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AE36" t="str">
-        <v/>
-      </c>
-      <c r="AF36" t="str">
-        <v/>
-      </c>
-      <c r="AG36" t="str">
-        <v>E</v>
-      </c>
-      <c r="AH36" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AI36">
-        <v>0</v>
-      </c>
-      <c r="AJ36">
-        <v>2</v>
-      </c>
-      <c r="AK36">
-        <v>6</v>
-      </c>
-      <c r="AL36">
-        <v>10</v>
-      </c>
-      <c r="AM36">
-        <v>0</v>
-      </c>
-      <c r="AN36">
         <v>216</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 09/2026 from web (22 NV)
</commit_message>
<xml_diff>
--- a/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
+++ b/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN35"/>
+  <dimension ref="A1:AN33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1407,7 +1407,7 @@
         <v/>
       </c>
       <c r="C18" t="str">
-        <v>Phan Như Ngọc</v>
+        <v>Nguyễn Phạm Quỳnh Trang</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -1523,19 +1523,19 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>DSP HDQ</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>30904</v>
       </c>
       <c r="C19" t="str">
-        <v>Nguyễn Phạm Quỳnh Trang</v>
+        <v>Trần Đình Đạt</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -1547,31 +1547,31 @@
         <v/>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K19" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="L19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O19" t="str">
         <v/>
       </c>
       <c r="P19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R19" t="str">
         <v/>
@@ -1580,22 +1580,22 @@
         <v/>
       </c>
       <c r="T19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V19" t="str">
         <v/>
       </c>
       <c r="W19" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="X19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z19" t="str">
         <v/>
@@ -1604,10 +1604,10 @@
         <v/>
       </c>
       <c r="AB19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD19" t="str">
         <v/>
@@ -1616,31 +1616,31 @@
         <v/>
       </c>
       <c r="AF19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH19" t="str">
         <v/>
       </c>
       <c r="AI19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AK19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AL19">
         <v>0</v>
       </c>
       <c r="AM19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN19">
-        <v>0</v>
+        <v>220</v>
       </c>
     </row>
     <row r="20">
@@ -1648,16 +1648,16 @@
         <v/>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>30905</v>
       </c>
       <c r="C20" t="str">
-        <v>Nguyễn Phương Linh</v>
+        <v>Nguyễn Trương Hoàng Hưng</v>
       </c>
       <c r="D20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -1666,22 +1666,22 @@
         <v/>
       </c>
       <c r="H20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="L20" t="str">
         <v/>
       </c>
       <c r="M20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N20" t="str">
         <v/>
@@ -1690,19 +1690,19 @@
         <v/>
       </c>
       <c r="P20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q20" t="str">
         <v/>
       </c>
       <c r="R20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="U20" t="str">
         <v/>
@@ -1711,19 +1711,19 @@
         <v/>
       </c>
       <c r="W20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="X20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y20" t="str">
         <v/>
       </c>
       <c r="Z20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB20" t="str">
         <v/>
@@ -1732,7 +1732,7 @@
         <v/>
       </c>
       <c r="AD20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE20" t="str">
         <v/>
@@ -1741,138 +1741,138 @@
         <v/>
       </c>
       <c r="AG20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AH20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AI20">
         <v>0</v>
       </c>
       <c r="AJ20">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AK20">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AL20">
         <v>0</v>
       </c>
       <c r="AM20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN20">
-        <v>0</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>DSP HDQ</v>
+        <v/>
       </c>
       <c r="B21" t="str">
-        <v>30904</v>
+        <v>30841</v>
       </c>
       <c r="C21" t="str">
-        <v>Trần Đình Đạt</v>
+        <v>Vũ Hoàng Long</v>
       </c>
       <c r="D21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="E21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="H21" t="str">
-        <v/>
+        <v>P</v>
       </c>
       <c r="I21" t="str">
-        <v>M</v>
+        <v>P</v>
       </c>
       <c r="J21" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="K21" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N21" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="O21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="U21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W21" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="X21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC21" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AD21" t="str">
         <v/>
       </c>
       <c r="AE21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AG21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AI21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ21">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AK21">
         <v>7</v>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="AN21">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22">
@@ -1892,112 +1892,112 @@
         <v/>
       </c>
       <c r="B22" t="str">
-        <v>30905</v>
+        <v>29718</v>
       </c>
       <c r="C22" t="str">
-        <v>Nguyễn Trương Hoàng Hưng</v>
+        <v>Vũ Huy Hùng</v>
       </c>
       <c r="D22" t="str">
-        <v>E</v>
+        <v>HC</v>
       </c>
       <c r="E22" t="str">
-        <v>E</v>
+        <v>HC</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="H22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I22" t="str">
-        <v>E</v>
+        <v>HC</v>
       </c>
       <c r="J22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="K22" t="str">
         <v>NL</v>
       </c>
       <c r="L22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N22" t="str">
         <v/>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="T22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="W22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="X22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC22" t="str">
         <v/>
       </c>
       <c r="AD22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AE22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF22" t="str">
         <v/>
       </c>
       <c r="AG22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AH22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AI22">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK22">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AL22">
         <v>0</v>
@@ -2006,60 +2006,60 @@
         <v>1</v>
       </c>
       <c r="AN22">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v/>
+        <v>DSP ASST HDQ</v>
       </c>
       <c r="B23" t="str">
-        <v>30841</v>
+        <v>39278</v>
       </c>
       <c r="C23" t="str">
-        <v>Vũ Hoàng Long</v>
+        <v>Nguyền Kiều Huyền Chi</v>
       </c>
       <c r="D23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E23" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G23" t="str">
         <v>M</v>
       </c>
       <c r="H23" t="str">
-        <v>P</v>
+        <v>E</v>
       </c>
       <c r="I23" t="str">
-        <v>P</v>
+        <v/>
       </c>
       <c r="J23" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="K23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="L23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M23" t="str">
         <v/>
       </c>
       <c r="N23" t="str">
-        <v>M</v>
+        <v>SN</v>
       </c>
       <c r="O23" t="str">
         <v>E</v>
       </c>
       <c r="P23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R23" t="str">
         <v>M</v>
@@ -2071,10 +2071,10 @@
         <v/>
       </c>
       <c r="U23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W23" t="str">
         <v>E</v>
@@ -2089,46 +2089,46 @@
         <v>M</v>
       </c>
       <c r="AA23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB23" t="str">
         <v/>
       </c>
       <c r="AC23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AF23" t="str">
-        <v>E</v>
+        <v>C349</v>
       </c>
       <c r="AG23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AH23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AI23">
         <v>0</v>
       </c>
       <c r="AJ23">
+        <v>8</v>
+      </c>
+      <c r="AK23">
         <v>9</v>
       </c>
-      <c r="AK23">
-        <v>7</v>
-      </c>
       <c r="AL23">
         <v>0</v>
       </c>
       <c r="AM23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN23">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="24">
@@ -2136,112 +2136,112 @@
         <v/>
       </c>
       <c r="B24" t="str">
-        <v>29718</v>
+        <v>39280</v>
       </c>
       <c r="C24" t="str">
-        <v>Vũ Huy Hùng</v>
+        <v>Đặng Thảo Linh</v>
       </c>
       <c r="D24" t="str">
+        <v/>
+      </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
+      <c r="F24" t="str">
+        <v>M</v>
+      </c>
+      <c r="G24" t="str">
+        <v>E</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v>E</v>
+      </c>
+      <c r="J24" t="str">
+        <v>NL</v>
+      </c>
+      <c r="K24" t="str">
+        <v>M</v>
+      </c>
+      <c r="L24" t="str">
+        <v>M</v>
+      </c>
+      <c r="M24" t="str">
+        <v>E</v>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v>M</v>
+      </c>
+      <c r="P24" t="str">
+        <v>E</v>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v>E</v>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v>M</v>
+      </c>
+      <c r="X24" t="str">
+        <v>M</v>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+      <c r="Z24" t="str">
         <v>HC</v>
       </c>
-      <c r="E24" t="str">
-        <v>HC</v>
-      </c>
-      <c r="F24" t="str">
-        <v>HC</v>
-      </c>
-      <c r="G24" t="str">
-        <v>HC</v>
-      </c>
-      <c r="H24" t="str">
-        <v/>
-      </c>
-      <c r="I24" t="str">
-        <v>HC</v>
-      </c>
-      <c r="J24" t="str">
-        <v>M</v>
-      </c>
-      <c r="K24" t="str">
-        <v>NL</v>
-      </c>
-      <c r="L24" t="str">
-        <v>E</v>
-      </c>
-      <c r="M24" t="str">
-        <v>E</v>
-      </c>
-      <c r="N24" t="str">
-        <v/>
-      </c>
-      <c r="O24" t="str">
-        <v>M</v>
-      </c>
-      <c r="P24" t="str">
-        <v/>
-      </c>
-      <c r="Q24" t="str">
-        <v>M</v>
-      </c>
-      <c r="R24" t="str">
-        <v>E</v>
-      </c>
-      <c r="S24" t="str">
-        <v/>
-      </c>
-      <c r="T24" t="str">
-        <v/>
-      </c>
-      <c r="U24" t="str">
-        <v>M</v>
-      </c>
-      <c r="V24" t="str">
-        <v>E</v>
-      </c>
-      <c r="W24" t="str">
-        <v/>
-      </c>
-      <c r="X24" t="str">
-        <v/>
-      </c>
-      <c r="Y24" t="str">
-        <v>M</v>
-      </c>
-      <c r="Z24" t="str">
-        <v>E</v>
-      </c>
       <c r="AA24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB24" t="str">
         <v>E</v>
       </c>
       <c r="AC24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AI24">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AJ24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AK24">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AL24">
         <v>0</v>
@@ -2250,90 +2250,90 @@
         <v>1</v>
       </c>
       <c r="AN24">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>DSP ASST HDQ</v>
+        <v/>
       </c>
       <c r="B25" t="str">
-        <v>39278</v>
+        <v>39276</v>
       </c>
       <c r="C25" t="str">
-        <v>Nguyền Kiều Huyền Chi</v>
+        <v>Bùi Việt Anh</v>
       </c>
       <c r="D25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="E25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F25" t="str">
         <v/>
       </c>
       <c r="G25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="H25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="I25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="K25" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="L25" t="str">
-        <v>E</v>
+        <v>P</v>
       </c>
       <c r="M25" t="str">
         <v/>
       </c>
       <c r="N25" t="str">
-        <v>SN</v>
+        <v>M</v>
       </c>
       <c r="O25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P25" t="str">
         <v/>
       </c>
       <c r="Q25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="S25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="T25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="V25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="X25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AA25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB25" t="str">
         <v/>
@@ -2342,37 +2342,37 @@
         <v/>
       </c>
       <c r="AD25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AE25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF25" t="str">
-        <v>C349</v>
+        <v/>
       </c>
       <c r="AG25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AH25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AI25">
         <v>0</v>
       </c>
       <c r="AJ25">
+        <v>9</v>
+      </c>
+      <c r="AK25">
         <v>8</v>
       </c>
-      <c r="AK25">
-        <v>9</v>
-      </c>
       <c r="AL25">
         <v>0</v>
       </c>
       <c r="AM25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN25">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26">
@@ -2380,109 +2380,109 @@
         <v/>
       </c>
       <c r="B26" t="str">
-        <v>39280</v>
+        <v>39274</v>
       </c>
       <c r="C26" t="str">
-        <v>Đặng Thảo Linh</v>
+        <v>Đỗ Nam Anh</v>
       </c>
       <c r="D26" t="str">
         <v/>
       </c>
       <c r="E26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="G26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="J26" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="K26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="L26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="N26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="P26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Q26" t="str">
         <v/>
       </c>
       <c r="R26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S26" t="str">
         <v/>
       </c>
       <c r="T26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="U26" t="str">
         <v/>
       </c>
       <c r="V26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z26" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="AA26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AC26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AD26" t="str">
         <v/>
       </c>
       <c r="AE26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AG26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AI26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ26">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK26">
         <v>9</v>
@@ -2491,36 +2491,36 @@
         <v>0</v>
       </c>
       <c r="AM26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN26">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v/>
+        <v>DSP SGN</v>
       </c>
       <c r="B27" t="str">
-        <v>39276</v>
+        <v>31844</v>
       </c>
       <c r="C27" t="str">
-        <v>Bùi Việt Anh</v>
+        <v>Nguyễn Hoàng Huy</v>
       </c>
       <c r="D27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="E27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G27" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="H27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I27" t="str">
         <v>E</v>
@@ -2532,13 +2532,13 @@
         <v>NL</v>
       </c>
       <c r="L27" t="str">
-        <v>P</v>
+        <v>M</v>
       </c>
       <c r="M27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="O27" t="str">
         <v/>
@@ -2547,13 +2547,13 @@
         <v/>
       </c>
       <c r="Q27" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="R27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="T27" t="str">
         <v>M</v>
@@ -2562,25 +2562,25 @@
         <v>E</v>
       </c>
       <c r="V27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="W27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="X27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y27" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Z27" t="str">
         <v/>
       </c>
       <c r="AA27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC27" t="str">
         <v/>
@@ -2589,10 +2589,10 @@
         <v>M</v>
       </c>
       <c r="AE27" t="str">
-        <v>E</v>
+        <v>HC</v>
       </c>
       <c r="AF27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG27" t="str">
         <v/>
@@ -2601,10 +2601,10 @@
         <v>M</v>
       </c>
       <c r="AI27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ27">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AK27">
         <v>8</v>
@@ -2616,7 +2616,7 @@
         <v>1</v>
       </c>
       <c r="AN27">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="28">
@@ -2624,40 +2624,40 @@
         <v/>
       </c>
       <c r="B28" t="str">
-        <v>39274</v>
+        <v>31843</v>
       </c>
       <c r="C28" t="str">
-        <v>Đỗ Nam Anh</v>
+        <v>Lương Trung Hiếu</v>
       </c>
       <c r="D28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="F28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="G28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="H28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J28" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="K28" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="L28" t="str">
         <v/>
       </c>
       <c r="M28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N28" t="str">
         <v>E</v>
@@ -2669,13 +2669,13 @@
         <v>M</v>
       </c>
       <c r="Q28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R28" t="str">
         <v/>
       </c>
       <c r="S28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T28" t="str">
         <v>E</v>
@@ -2684,28 +2684,28 @@
         <v/>
       </c>
       <c r="V28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="W28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="X28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AD28" t="str">
         <v/>
@@ -2714,28 +2714,28 @@
         <v>M</v>
       </c>
       <c r="AF28" t="str">
-        <v>E</v>
+        <v>HC</v>
       </c>
       <c r="AG28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH28" t="str">
         <v/>
       </c>
       <c r="AI28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ28">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AK28">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AL28">
         <v>0</v>
       </c>
       <c r="AM28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AN28">
         <v>216</v>
@@ -2743,124 +2743,124 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>DSP SGN</v>
+        <v/>
       </c>
       <c r="B29" t="str">
-        <v>31844</v>
+        <v>31846</v>
       </c>
       <c r="C29" t="str">
-        <v>Nguyễn Hoàng Huy</v>
+        <v>Nguyễn Phúc Thịnh</v>
       </c>
       <c r="D29" t="str">
         <v>E</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G29" t="str">
-        <v>SN</v>
+        <v>M</v>
       </c>
       <c r="H29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="K29" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="N29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="R29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="S29" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="T29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="U29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W29" t="str">
         <v/>
       </c>
       <c r="X29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Z29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AE29" t="str">
+        <v/>
+      </c>
+      <c r="AF29" t="str">
+        <v>M</v>
+      </c>
+      <c r="AG29" t="str">
         <v>HC</v>
       </c>
-      <c r="AF29" t="str">
-        <v>E</v>
-      </c>
-      <c r="AG29" t="str">
-        <v/>
-      </c>
       <c r="AH29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AI29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ29">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK29">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AL29">
         <v>0</v>
       </c>
       <c r="AM29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN29">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="30">
@@ -2868,106 +2868,106 @@
         <v/>
       </c>
       <c r="B30" t="str">
-        <v>31843</v>
+        <v>31847</v>
       </c>
       <c r="C30" t="str">
-        <v>Lương Trung Hiếu</v>
+        <v>Hoàng Bảo Ngọc</v>
       </c>
       <c r="D30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="E30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J30" t="str">
         <v>NL</v>
       </c>
       <c r="K30" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="L30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N30" t="str">
         <v>E</v>
       </c>
       <c r="O30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R30" t="str">
         <v/>
       </c>
       <c r="S30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AA30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC30" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AD30" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="AE30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF30" t="str">
+        <v/>
+      </c>
+      <c r="AG30" t="str">
+        <v>M</v>
+      </c>
+      <c r="AH30" t="str">
         <v>HC</v>
       </c>
-      <c r="AG30" t="str">
-        <v>E</v>
-      </c>
-      <c r="AH30" t="str">
-        <v/>
-      </c>
       <c r="AI30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ30">
         <v>8</v>
@@ -2979,7 +2979,7 @@
         <v>0</v>
       </c>
       <c r="AM30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN30">
         <v>216</v>
@@ -2987,61 +2987,61 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>DSP PQC</v>
       </c>
       <c r="B31" t="str">
-        <v>31846</v>
+        <v>41863</v>
       </c>
       <c r="C31" t="str">
-        <v>Nguyễn Phúc Thịnh</v>
+        <v>Lê Ngọc Thành Tài</v>
       </c>
       <c r="D31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E31" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="G31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="H31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="I31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="J31" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="K31" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="L31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M31" t="str">
         <v/>
       </c>
       <c r="N31" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="O31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="P31" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Q31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="R31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="S31" t="str">
-        <v>HC</v>
+        <v>C9</v>
       </c>
       <c r="T31" t="str">
         <v/>
@@ -3050,61 +3050,61 @@
         <v/>
       </c>
       <c r="V31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="W31" t="str">
         <v/>
       </c>
       <c r="X31" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Y31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Z31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AC31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG31" t="str">
-        <v>HC</v>
+        <v>C9</v>
       </c>
       <c r="AH31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AI31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ31">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AK31">
+        <v>4</v>
+      </c>
+      <c r="AL31">
         <v>10</v>
       </c>
-      <c r="AL31">
-        <v>0</v>
-      </c>
       <c r="AM31">
         <v>0</v>
       </c>
       <c r="AN31">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="32">
@@ -3112,118 +3112,118 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>31847</v>
+        <v>41865</v>
       </c>
       <c r="C32" t="str">
-        <v>Hoàng Bảo Ngọc</v>
+        <v>Nguyễn Đức Lộc</v>
       </c>
       <c r="D32" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="E32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="G32" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="H32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J32" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="K32" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="L32" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="M32" t="str">
         <v/>
       </c>
       <c r="N32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O32" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="P32" t="str">
         <v/>
       </c>
       <c r="Q32" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R32" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="S32" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T32" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="U32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="V32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="W32" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="X32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y32" t="str">
         <v/>
       </c>
       <c r="Z32" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AA32" t="str">
         <v/>
       </c>
       <c r="AB32" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC32" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="AD32" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AE32" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="AF32" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AG32" t="str">
         <v>M</v>
       </c>
       <c r="AH32" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AI32">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ32">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AK32">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="AL32">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AM32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN32">
         <v>216</v>
@@ -3231,115 +3231,115 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>DSP PQC</v>
+        <v/>
       </c>
       <c r="B33" t="str">
-        <v>41863</v>
+        <v>41867</v>
       </c>
       <c r="C33" t="str">
-        <v>Lê Ngọc Thành Tài</v>
+        <v>Phan Thành Nghĩa</v>
       </c>
       <c r="D33" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E33" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
         <v>C9</v>
       </c>
-      <c r="G33" t="str">
-        <v>E</v>
-      </c>
-      <c r="H33" t="str">
-        <v/>
-      </c>
       <c r="I33" t="str">
+        <v>E</v>
+      </c>
+      <c r="J33" t="str">
+        <v>E</v>
+      </c>
+      <c r="K33" t="str">
+        <v>E</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
         <v>C9</v>
       </c>
-      <c r="J33" t="str">
+      <c r="N33" t="str">
+        <v>E</v>
+      </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
+      <c r="P33" t="str">
         <v>C9</v>
       </c>
-      <c r="K33" t="str">
-        <v>M</v>
-      </c>
-      <c r="L33" t="str">
-        <v>E</v>
-      </c>
-      <c r="M33" t="str">
-        <v/>
-      </c>
-      <c r="N33" t="str">
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
         <v>C9</v>
       </c>
-      <c r="O33" t="str">
-        <v/>
-      </c>
-      <c r="P33" t="str">
-        <v>M</v>
-      </c>
-      <c r="Q33" t="str">
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v>M</v>
+      </c>
+      <c r="X33" t="str">
         <v>C9</v>
       </c>
-      <c r="R33" t="str">
-        <v/>
-      </c>
-      <c r="S33" t="str">
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
         <v>C9</v>
       </c>
-      <c r="T33" t="str">
-        <v/>
-      </c>
-      <c r="U33" t="str">
-        <v/>
-      </c>
-      <c r="V33" t="str">
+      <c r="AA33" t="str">
         <v>C9</v>
       </c>
-      <c r="W33" t="str">
-        <v/>
-      </c>
-      <c r="X33" t="str">
-        <v>M</v>
-      </c>
-      <c r="Y33" t="str">
+      <c r="AB33" t="str">
+        <v>E</v>
+      </c>
+      <c r="AC33" t="str">
+        <v/>
+      </c>
+      <c r="AD33" t="str">
         <v>C9</v>
       </c>
-      <c r="Z33" t="str">
-        <v>E</v>
-      </c>
-      <c r="AA33" t="str">
-        <v/>
-      </c>
-      <c r="AB33" t="str">
+      <c r="AE33" t="str">
+        <v/>
+      </c>
+      <c r="AF33" t="str">
+        <v/>
+      </c>
+      <c r="AG33" t="str">
+        <v>E</v>
+      </c>
+      <c r="AH33" t="str">
         <v>C9</v>
       </c>
-      <c r="AC33" t="str">
-        <v/>
-      </c>
-      <c r="AD33" t="str">
-        <v/>
-      </c>
-      <c r="AE33" t="str">
-        <v>E</v>
-      </c>
-      <c r="AF33" t="str">
-        <v/>
-      </c>
-      <c r="AG33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AH33" t="str">
-        <v/>
-      </c>
       <c r="AI33">
         <v>0</v>
       </c>
       <c r="AJ33">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AK33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AL33">
         <v>10</v>
@@ -3348,256 +3348,12 @@
         <v>0</v>
       </c>
       <c r="AN33">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v/>
-      </c>
-      <c r="B34" t="str">
-        <v>41865</v>
-      </c>
-      <c r="C34" t="str">
-        <v>Nguyễn Đức Lộc</v>
-      </c>
-      <c r="D34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="E34" t="str">
-        <v>E</v>
-      </c>
-      <c r="F34" t="str">
-        <v/>
-      </c>
-      <c r="G34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="H34" t="str">
-        <v/>
-      </c>
-      <c r="I34" t="str">
-        <v/>
-      </c>
-      <c r="J34" t="str">
-        <v>M</v>
-      </c>
-      <c r="K34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="L34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="M34" t="str">
-        <v/>
-      </c>
-      <c r="N34" t="str">
-        <v/>
-      </c>
-      <c r="O34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="P34" t="str">
-        <v/>
-      </c>
-      <c r="Q34" t="str">
-        <v>M</v>
-      </c>
-      <c r="R34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="S34" t="str">
-        <v/>
-      </c>
-      <c r="T34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="U34" t="str">
-        <v>E</v>
-      </c>
-      <c r="V34" t="str">
-        <v/>
-      </c>
-      <c r="W34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="X34" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y34" t="str">
-        <v/>
-      </c>
-      <c r="Z34" t="str">
-        <v>M</v>
-      </c>
-      <c r="AA34" t="str">
-        <v/>
-      </c>
-      <c r="AB34" t="str">
-        <v/>
-      </c>
-      <c r="AC34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AD34" t="str">
-        <v/>
-      </c>
-      <c r="AE34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AF34" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AG34" t="str">
-        <v>M</v>
-      </c>
-      <c r="AH34" t="str">
-        <v/>
-      </c>
-      <c r="AI34">
-        <v>0</v>
-      </c>
-      <c r="AJ34">
-        <v>4</v>
-      </c>
-      <c r="AK34">
-        <v>3</v>
-      </c>
-      <c r="AL34">
-        <v>11</v>
-      </c>
-      <c r="AM34">
-        <v>0</v>
-      </c>
-      <c r="AN34">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v/>
-      </c>
-      <c r="B35" t="str">
-        <v>41867</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Phan Thành Nghĩa</v>
-      </c>
-      <c r="D35" t="str">
-        <v>M</v>
-      </c>
-      <c r="E35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="F35" t="str">
-        <v/>
-      </c>
-      <c r="G35" t="str">
-        <v/>
-      </c>
-      <c r="H35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="I35" t="str">
-        <v>E</v>
-      </c>
-      <c r="J35" t="str">
-        <v>E</v>
-      </c>
-      <c r="K35" t="str">
-        <v>E</v>
-      </c>
-      <c r="L35" t="str">
-        <v/>
-      </c>
-      <c r="M35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="N35" t="str">
-        <v>E</v>
-      </c>
-      <c r="O35" t="str">
-        <v/>
-      </c>
-      <c r="P35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="Q35" t="str">
-        <v/>
-      </c>
-      <c r="R35" t="str">
-        <v/>
-      </c>
-      <c r="S35" t="str">
-        <v/>
-      </c>
-      <c r="T35" t="str">
-        <v/>
-      </c>
-      <c r="U35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="V35" t="str">
-        <v/>
-      </c>
-      <c r="W35" t="str">
-        <v>M</v>
-      </c>
-      <c r="X35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="Y35" t="str">
-        <v/>
-      </c>
-      <c r="Z35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AA35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AB35" t="str">
-        <v>E</v>
-      </c>
-      <c r="AC35" t="str">
-        <v/>
-      </c>
-      <c r="AD35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AE35" t="str">
-        <v/>
-      </c>
-      <c r="AF35" t="str">
-        <v/>
-      </c>
-      <c r="AG35" t="str">
-        <v>E</v>
-      </c>
-      <c r="AH35" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AI35">
-        <v>0</v>
-      </c>
-      <c r="AJ35">
-        <v>2</v>
-      </c>
-      <c r="AK35">
-        <v>6</v>
-      </c>
-      <c r="AL35">
-        <v>10</v>
-      </c>
-      <c r="AM35">
-        <v>0</v>
-      </c>
-      <c r="AN35">
         <v>216</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 09/2026 from web (23 NV)
</commit_message>
<xml_diff>
--- a/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
+++ b/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN33"/>
+  <dimension ref="A1:AN34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1407,7 +1407,7 @@
         <v/>
       </c>
       <c r="C18" t="str">
-        <v>Nguyễn Phạm Quỳnh Trang</v>
+        <v>Phan Như Ngọc</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -1523,19 +1523,19 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>DSP HDQ</v>
+        <v/>
       </c>
       <c r="B19" t="str">
-        <v>30904</v>
+        <v/>
       </c>
       <c r="C19" t="str">
-        <v>Trần Đình Đạt</v>
+        <v>Nguyễn Phương Linh</v>
       </c>
       <c r="D19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="E19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -1547,31 +1547,31 @@
         <v/>
       </c>
       <c r="I19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="K19" t="str">
-        <v>NL</v>
+        <v/>
       </c>
       <c r="L19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O19" t="str">
         <v/>
       </c>
       <c r="P19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R19" t="str">
         <v/>
@@ -1580,22 +1580,22 @@
         <v/>
       </c>
       <c r="T19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="U19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V19" t="str">
         <v/>
       </c>
       <c r="W19" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="X19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z19" t="str">
         <v/>
@@ -1604,10 +1604,10 @@
         <v/>
       </c>
       <c r="AB19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD19" t="str">
         <v/>
@@ -1616,48 +1616,48 @@
         <v/>
       </c>
       <c r="AF19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH19" t="str">
         <v/>
       </c>
       <c r="AI19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ19">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AK19">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="AL19">
         <v>0</v>
       </c>
       <c r="AM19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN19">
-        <v>220</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>DSP HDQ</v>
       </c>
       <c r="B20" t="str">
-        <v>30905</v>
+        <v>30904</v>
       </c>
       <c r="C20" t="str">
-        <v>Nguyễn Trương Hoàng Hưng</v>
+        <v>Trần Đình Đạt</v>
       </c>
       <c r="D20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="E20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -1666,94 +1666,94 @@
         <v/>
       </c>
       <c r="H20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="J20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="K20" t="str">
         <v>NL</v>
       </c>
       <c r="L20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M20" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O20" t="str">
         <v/>
       </c>
       <c r="P20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Q20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="S20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="T20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="U20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V20" t="str">
         <v/>
       </c>
       <c r="W20" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="X20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Y20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AA20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE20" t="str">
         <v/>
       </c>
       <c r="AF20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG20" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AH20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AI20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ20">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AK20">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AL20">
         <v>0</v>
@@ -1762,7 +1762,7 @@
         <v>1</v>
       </c>
       <c r="AN20">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21">
@@ -1770,46 +1770,46 @@
         <v/>
       </c>
       <c r="B21" t="str">
-        <v>30841</v>
+        <v>30905</v>
       </c>
       <c r="C21" t="str">
-        <v>Vũ Hoàng Long</v>
+        <v>Nguyễn Trương Hoàng Hưng</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="H21" t="str">
-        <v>P</v>
+        <v>M</v>
       </c>
       <c r="I21" t="str">
-        <v>P</v>
+        <v>E</v>
       </c>
       <c r="J21" t="str">
+        <v>E</v>
+      </c>
+      <c r="K21" t="str">
         <v>NL</v>
       </c>
-      <c r="K21" t="str">
-        <v>E</v>
-      </c>
       <c r="L21" t="str">
         <v/>
       </c>
       <c r="M21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="O21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P21" t="str">
         <v>E</v>
@@ -1821,22 +1821,22 @@
         <v>M</v>
       </c>
       <c r="S21" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="T21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="U21" t="str">
         <v/>
       </c>
       <c r="V21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="W21" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="X21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y21" t="str">
         <v/>
@@ -1845,37 +1845,37 @@
         <v>M</v>
       </c>
       <c r="AA21" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AB21" t="str">
         <v/>
       </c>
       <c r="AC21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AF21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AG21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AH21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AI21">
         <v>0</v>
       </c>
       <c r="AJ21">
+        <v>8</v>
+      </c>
+      <c r="AK21">
         <v>9</v>
-      </c>
-      <c r="AK21">
-        <v>7</v>
       </c>
       <c r="AL21">
         <v>0</v>
@@ -1884,7 +1884,7 @@
         <v>1</v>
       </c>
       <c r="AN21">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22">
@@ -1892,97 +1892,97 @@
         <v/>
       </c>
       <c r="B22" t="str">
-        <v>29718</v>
+        <v>30841</v>
       </c>
       <c r="C22" t="str">
-        <v>Vũ Huy Hùng</v>
+        <v>Vũ Hoàng Long</v>
       </c>
       <c r="D22" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="E22" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="G22" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>P</v>
       </c>
       <c r="I22" t="str">
-        <v>HC</v>
+        <v>P</v>
       </c>
       <c r="J22" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="K22" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="R22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="S22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T22" t="str">
         <v/>
       </c>
       <c r="U22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="W22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X22" t="str">
         <v/>
       </c>
       <c r="Y22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Z22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AA22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AF22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG22" t="str">
         <v/>
@@ -1991,10 +1991,10 @@
         <v>M</v>
       </c>
       <c r="AI22">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ22">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AK22">
         <v>7</v>
@@ -2011,49 +2011,49 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>DSP ASST HDQ</v>
+        <v/>
       </c>
       <c r="B23" t="str">
-        <v>39278</v>
+        <v>29718</v>
       </c>
       <c r="C23" t="str">
-        <v>Nguyền Kiều Huyền Chi</v>
+        <v>Vũ Huy Hùng</v>
       </c>
       <c r="D23" t="str">
-        <v>E</v>
+        <v>HC</v>
       </c>
       <c r="E23" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="G23" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="H23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="I23" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="J23" t="str">
         <v>M</v>
       </c>
       <c r="K23" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="L23" t="str">
         <v>E</v>
       </c>
       <c r="M23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N23" t="str">
-        <v>SN</v>
+        <v/>
       </c>
       <c r="O23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="P23" t="str">
         <v/>
@@ -2062,10 +2062,10 @@
         <v>M</v>
       </c>
       <c r="R23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T23" t="str">
         <v/>
@@ -2077,165 +2077,165 @@
         <v>E</v>
       </c>
       <c r="W23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X23" t="str">
         <v/>
       </c>
       <c r="Y23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA23" t="str">
         <v/>
       </c>
       <c r="AB23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC23" t="str">
         <v/>
       </c>
       <c r="AD23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AE23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF23" t="str">
-        <v>C349</v>
+        <v/>
       </c>
       <c r="AG23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AH23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AI23">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ23">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK23">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AL23">
         <v>0</v>
       </c>
       <c r="AM23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN23">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v/>
+        <v>DSP ASST HDQ</v>
       </c>
       <c r="B24" t="str">
-        <v>39280</v>
+        <v>39278</v>
       </c>
       <c r="C24" t="str">
-        <v>Đặng Thảo Linh</v>
+        <v>Nguyền Kiều Huyền Chi</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E24" t="str">
         <v/>
       </c>
       <c r="F24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G24" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J24" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="K24" t="str">
         <v>M</v>
       </c>
       <c r="L24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="M24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="O24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R24" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="S24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T24" t="str">
         <v/>
       </c>
       <c r="U24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="W24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y24" t="str">
         <v/>
       </c>
       <c r="Z24" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="AA24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE24" t="str">
         <v/>
       </c>
       <c r="AF24" t="str">
-        <v>M</v>
+        <v>C349</v>
       </c>
       <c r="AG24" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AH24" t="str">
         <v>E</v>
       </c>
       <c r="AI24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ24">
         <v>8</v>
@@ -2247,10 +2247,10 @@
         <v>0</v>
       </c>
       <c r="AM24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN24">
-        <v>220</v>
+        <v>212</v>
       </c>
     </row>
     <row r="25">
@@ -2258,64 +2258,64 @@
         <v/>
       </c>
       <c r="B25" t="str">
-        <v>39276</v>
+        <v>39280</v>
       </c>
       <c r="C25" t="str">
-        <v>Bùi Việt Anh</v>
+        <v>Đặng Thảo Linh</v>
       </c>
       <c r="D25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="E25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="H25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I25" t="str">
         <v>E</v>
       </c>
       <c r="J25" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="K25" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="L25" t="str">
-        <v>P</v>
+        <v>M</v>
       </c>
       <c r="M25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="O25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="T25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="U25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V25" t="str">
         <v/>
@@ -2324,46 +2324,46 @@
         <v>M</v>
       </c>
       <c r="X25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Y25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z25" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="AA25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AB25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AI25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ25">
+        <v>8</v>
+      </c>
+      <c r="AK25">
         <v>9</v>
-      </c>
-      <c r="AK25">
-        <v>8</v>
       </c>
       <c r="AL25">
         <v>0</v>
@@ -2380,19 +2380,19 @@
         <v/>
       </c>
       <c r="B26" t="str">
-        <v>39274</v>
+        <v>39276</v>
       </c>
       <c r="C26" t="str">
-        <v>Đỗ Nam Anh</v>
+        <v>Bùi Việt Anh</v>
       </c>
       <c r="D26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="F26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="G26" t="str">
         <v/>
@@ -2401,82 +2401,82 @@
         <v>M</v>
       </c>
       <c r="I26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="J26" t="str">
         <v>E</v>
       </c>
       <c r="K26" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="L26" t="str">
-        <v/>
+        <v>P</v>
       </c>
       <c r="M26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="N26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="O26" t="str">
         <v/>
       </c>
       <c r="P26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R26" t="str">
         <v/>
       </c>
       <c r="S26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="U26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="W26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="X26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AG26" t="str">
         <v/>
       </c>
       <c r="AH26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AI26">
         <v>0</v>
@@ -2485,87 +2485,87 @@
         <v>9</v>
       </c>
       <c r="AK26">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AL26">
         <v>0</v>
       </c>
       <c r="AM26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN26">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>DSP SGN</v>
+        <v/>
       </c>
       <c r="B27" t="str">
-        <v>31844</v>
+        <v>39274</v>
       </c>
       <c r="C27" t="str">
-        <v>Nguyễn Hoàng Huy</v>
+        <v>Đỗ Nam Anh</v>
       </c>
       <c r="D27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="G27" t="str">
-        <v>SN</v>
+        <v/>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I27" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="J27" t="str">
         <v>E</v>
       </c>
       <c r="K27" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M27" t="str">
         <v>M</v>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O27" t="str">
         <v/>
       </c>
       <c r="P27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="R27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S27" t="str">
         <v/>
       </c>
       <c r="T27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V27" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="W27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X27" t="str">
         <v/>
@@ -2574,22 +2574,22 @@
         <v>M</v>
       </c>
       <c r="Z27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AA27" t="str">
         <v/>
       </c>
       <c r="AB27" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AC27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE27" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="AF27" t="str">
         <v>E</v>
@@ -2598,22 +2598,22 @@
         <v/>
       </c>
       <c r="AH27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AI27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ27">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK27">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AL27">
         <v>0</v>
       </c>
       <c r="AM27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN27">
         <v>216</v>
@@ -2621,106 +2621,106 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v/>
+        <v>DSP SGN</v>
       </c>
       <c r="B28" t="str">
-        <v>31843</v>
+        <v>31844</v>
       </c>
       <c r="C28" t="str">
-        <v>Lương Trung Hiếu</v>
+        <v>Nguyễn Hoàng Huy</v>
       </c>
       <c r="D28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="E28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G28" t="str">
-        <v>E</v>
+        <v>SN</v>
       </c>
       <c r="H28" t="str">
         <v/>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J28" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="K28" t="str">
         <v>NL</v>
       </c>
       <c r="L28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="N28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O28" t="str">
         <v/>
       </c>
       <c r="P28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="R28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="T28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="U28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="W28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="X28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Z28" t="str">
         <v/>
       </c>
       <c r="AA28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AB28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE28" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="AF28" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="AG28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AI28">
         <v>1</v>
@@ -2735,7 +2735,7 @@
         <v>0</v>
       </c>
       <c r="AM28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN28">
         <v>216</v>
@@ -2746,121 +2746,121 @@
         <v/>
       </c>
       <c r="B29" t="str">
-        <v>31846</v>
+        <v>31843</v>
       </c>
       <c r="C29" t="str">
-        <v>Nguyễn Phúc Thịnh</v>
+        <v>Lương Trung Hiếu</v>
       </c>
       <c r="D29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="E29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="F29" t="str">
         <v/>
       </c>
       <c r="G29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="H29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="I29" t="str">
         <v/>
       </c>
       <c r="J29" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="K29" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="L29" t="str">
         <v/>
       </c>
       <c r="M29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="P29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Q29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="S29" t="str">
+        <v>M</v>
+      </c>
+      <c r="T29" t="str">
+        <v>E</v>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
+      <c r="W29" t="str">
+        <v>M</v>
+      </c>
+      <c r="X29" t="str">
+        <v>M</v>
+      </c>
+      <c r="Y29" t="str">
+        <v>E</v>
+      </c>
+      <c r="Z29" t="str">
+        <v/>
+      </c>
+      <c r="AA29" t="str">
+        <v>M</v>
+      </c>
+      <c r="AB29" t="str">
+        <v/>
+      </c>
+      <c r="AC29" t="str">
+        <v>E</v>
+      </c>
+      <c r="AD29" t="str">
+        <v/>
+      </c>
+      <c r="AE29" t="str">
+        <v>M</v>
+      </c>
+      <c r="AF29" t="str">
         <v>HC</v>
       </c>
-      <c r="T29" t="str">
-        <v/>
-      </c>
-      <c r="U29" t="str">
-        <v/>
-      </c>
-      <c r="V29" t="str">
-        <v/>
-      </c>
-      <c r="W29" t="str">
-        <v/>
-      </c>
-      <c r="X29" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y29" t="str">
-        <v/>
-      </c>
-      <c r="Z29" t="str">
-        <v>M</v>
-      </c>
-      <c r="AA29" t="str">
-        <v>E</v>
-      </c>
-      <c r="AB29" t="str">
-        <v/>
-      </c>
-      <c r="AC29" t="str">
-        <v>E</v>
-      </c>
-      <c r="AD29" t="str">
-        <v>E</v>
-      </c>
-      <c r="AE29" t="str">
-        <v/>
-      </c>
-      <c r="AF29" t="str">
-        <v>M</v>
-      </c>
       <c r="AG29" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="AH29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AI29">
+        <v>1</v>
+      </c>
+      <c r="AJ29">
+        <v>8</v>
+      </c>
+      <c r="AK29">
+        <v>8</v>
+      </c>
+      <c r="AL29">
+        <v>0</v>
+      </c>
+      <c r="AM29">
         <v>2</v>
       </c>
-      <c r="AJ29">
-        <v>7</v>
-      </c>
-      <c r="AK29">
-        <v>10</v>
-      </c>
-      <c r="AL29">
-        <v>0</v>
-      </c>
-      <c r="AM29">
-        <v>0</v>
-      </c>
       <c r="AN29">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="30">
@@ -2868,153 +2868,153 @@
         <v/>
       </c>
       <c r="B30" t="str">
-        <v>31847</v>
+        <v>31846</v>
       </c>
       <c r="C30" t="str">
-        <v>Hoàng Bảo Ngọc</v>
+        <v>Nguyễn Phúc Thịnh</v>
       </c>
       <c r="D30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="F30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="G30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="H30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="I30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="J30" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="K30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="L30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="M30" t="str">
         <v/>
       </c>
       <c r="N30" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="O30" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="P30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q30" t="str">
         <v/>
       </c>
       <c r="R30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S30" t="str">
-        <v>E</v>
+        <v>HC</v>
       </c>
       <c r="T30" t="str">
         <v/>
       </c>
       <c r="U30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="W30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Y30" t="str">
         <v/>
       </c>
       <c r="Z30" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AA30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AB30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC30" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AD30" t="str">
+        <v>E</v>
+      </c>
+      <c r="AE30" t="str">
+        <v/>
+      </c>
+      <c r="AF30" t="str">
+        <v>M</v>
+      </c>
+      <c r="AG30" t="str">
         <v>HC</v>
       </c>
-      <c r="AE30" t="str">
-        <v>E</v>
-      </c>
-      <c r="AF30" t="str">
-        <v/>
-      </c>
-      <c r="AG30" t="str">
-        <v>M</v>
-      </c>
       <c r="AH30" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="AI30">
         <v>2</v>
       </c>
       <c r="AJ30">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK30">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AL30">
         <v>0</v>
       </c>
       <c r="AM30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN30">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>DSP PQC</v>
+        <v/>
       </c>
       <c r="B31" t="str">
-        <v>41863</v>
+        <v>31847</v>
       </c>
       <c r="C31" t="str">
-        <v>Lê Ngọc Thành Tài</v>
+        <v>Hoàng Bảo Ngọc</v>
       </c>
       <c r="D31" t="str">
         <v/>
       </c>
       <c r="E31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="F31" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="G31" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="H31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I31" t="str">
-        <v>C9</v>
+        <v>M</v>
       </c>
       <c r="J31" t="str">
-        <v>C9</v>
+        <v>NL</v>
       </c>
       <c r="K31" t="str">
         <v>M</v>
@@ -3026,40 +3026,40 @@
         <v/>
       </c>
       <c r="N31" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="O31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q31" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="R31" t="str">
         <v/>
       </c>
       <c r="S31" t="str">
-        <v>C9</v>
+        <v>E</v>
       </c>
       <c r="T31" t="str">
         <v/>
       </c>
       <c r="U31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V31" t="str">
-        <v>C9</v>
+        <v>M</v>
       </c>
       <c r="W31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Y31" t="str">
-        <v>C9</v>
+        <v/>
       </c>
       <c r="Z31" t="str">
         <v>E</v>
@@ -3068,13 +3068,13 @@
         <v/>
       </c>
       <c r="AB31" t="str">
-        <v>C9</v>
+        <v>M</v>
       </c>
       <c r="AC31" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD31" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="AE31" t="str">
         <v>E</v>
@@ -3083,25 +3083,25 @@
         <v/>
       </c>
       <c r="AG31" t="str">
-        <v>C9</v>
+        <v>M</v>
       </c>
       <c r="AH31" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="AI31">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ31">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AK31">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="AL31">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AM31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN31">
         <v>216</v>
@@ -3109,103 +3109,103 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v/>
+        <v>DSP PQC</v>
       </c>
       <c r="B32" t="str">
-        <v>41865</v>
+        <v>41863</v>
       </c>
       <c r="C32" t="str">
-        <v>Nguyễn Đức Lộc</v>
+        <v>Lê Ngọc Thành Tài</v>
       </c>
       <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v>M</v>
+      </c>
+      <c r="F32" t="str">
         <v>C9</v>
       </c>
-      <c r="E32" t="str">
-        <v>E</v>
-      </c>
-      <c r="F32" t="str">
-        <v/>
-      </c>
       <c r="G32" t="str">
+        <v>E</v>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
         <v>C9</v>
       </c>
-      <c r="H32" t="str">
-        <v/>
-      </c>
-      <c r="I32" t="str">
-        <v/>
-      </c>
       <c r="J32" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="K32" t="str">
+        <v>M</v>
+      </c>
+      <c r="L32" t="str">
+        <v>E</v>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
         <v>C9</v>
       </c>
-      <c r="L32" t="str">
+      <c r="O32" t="str">
+        <v/>
+      </c>
+      <c r="P32" t="str">
+        <v>M</v>
+      </c>
+      <c r="Q32" t="str">
         <v>C9</v>
       </c>
-      <c r="M32" t="str">
-        <v/>
-      </c>
-      <c r="N32" t="str">
-        <v/>
-      </c>
-      <c r="O32" t="str">
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
         <v>C9</v>
       </c>
-      <c r="P32" t="str">
-        <v/>
-      </c>
-      <c r="Q32" t="str">
-        <v>M</v>
-      </c>
-      <c r="R32" t="str">
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
+        <v/>
+      </c>
+      <c r="V32" t="str">
         <v>C9</v>
       </c>
-      <c r="S32" t="str">
-        <v/>
-      </c>
-      <c r="T32" t="str">
+      <c r="W32" t="str">
+        <v/>
+      </c>
+      <c r="X32" t="str">
+        <v>M</v>
+      </c>
+      <c r="Y32" t="str">
         <v>C9</v>
       </c>
-      <c r="U32" t="str">
-        <v>E</v>
-      </c>
-      <c r="V32" t="str">
-        <v/>
-      </c>
-      <c r="W32" t="str">
+      <c r="Z32" t="str">
+        <v>E</v>
+      </c>
+      <c r="AA32" t="str">
+        <v/>
+      </c>
+      <c r="AB32" t="str">
         <v>C9</v>
       </c>
-      <c r="X32" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y32" t="str">
-        <v/>
-      </c>
-      <c r="Z32" t="str">
-        <v>M</v>
-      </c>
-      <c r="AA32" t="str">
-        <v/>
-      </c>
-      <c r="AB32" t="str">
-        <v/>
-      </c>
       <c r="AC32" t="str">
+        <v/>
+      </c>
+      <c r="AD32" t="str">
+        <v/>
+      </c>
+      <c r="AE32" t="str">
+        <v>E</v>
+      </c>
+      <c r="AF32" t="str">
+        <v/>
+      </c>
+      <c r="AG32" t="str">
         <v>C9</v>
-      </c>
-      <c r="AD32" t="str">
-        <v/>
-      </c>
-      <c r="AE32" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AF32" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AG32" t="str">
-        <v>M</v>
       </c>
       <c r="AH32" t="str">
         <v/>
@@ -3217,10 +3217,10 @@
         <v>4</v>
       </c>
       <c r="AK32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AL32">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AM32">
         <v>0</v>
@@ -3234,126 +3234,248 @@
         <v/>
       </c>
       <c r="B33" t="str">
+        <v>41865</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Nguyễn Đức Lộc</v>
+      </c>
+      <c r="D33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="E33" t="str">
+        <v>E</v>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v>M</v>
+      </c>
+      <c r="K33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="L33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v>M</v>
+      </c>
+      <c r="R33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="U33" t="str">
+        <v>E</v>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="X33" t="str">
+        <v>E</v>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v>M</v>
+      </c>
+      <c r="AA33" t="str">
+        <v/>
+      </c>
+      <c r="AB33" t="str">
+        <v/>
+      </c>
+      <c r="AC33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AD33" t="str">
+        <v/>
+      </c>
+      <c r="AE33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AF33" t="str">
+        <v>C9</v>
+      </c>
+      <c r="AG33" t="str">
+        <v>M</v>
+      </c>
+      <c r="AH33" t="str">
+        <v/>
+      </c>
+      <c r="AI33">
+        <v>0</v>
+      </c>
+      <c r="AJ33">
+        <v>4</v>
+      </c>
+      <c r="AK33">
+        <v>3</v>
+      </c>
+      <c r="AL33">
+        <v>11</v>
+      </c>
+      <c r="AM33">
+        <v>0</v>
+      </c>
+      <c r="AN33">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
         <v>41867</v>
       </c>
-      <c r="C33" t="str">
+      <c r="C34" t="str">
         <v>Phan Thành Nghĩa</v>
       </c>
-      <c r="D33" t="str">
-        <v>M</v>
-      </c>
-      <c r="E33" t="str">
+      <c r="D34" t="str">
+        <v>M</v>
+      </c>
+      <c r="E34" t="str">
         <v>C9</v>
       </c>
-      <c r="F33" t="str">
-        <v/>
-      </c>
-      <c r="G33" t="str">
-        <v/>
-      </c>
-      <c r="H33" t="str">
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
         <v>C9</v>
       </c>
-      <c r="I33" t="str">
-        <v>E</v>
-      </c>
-      <c r="J33" t="str">
-        <v>E</v>
-      </c>
-      <c r="K33" t="str">
-        <v>E</v>
-      </c>
-      <c r="L33" t="str">
-        <v/>
-      </c>
-      <c r="M33" t="str">
+      <c r="I34" t="str">
+        <v>E</v>
+      </c>
+      <c r="J34" t="str">
+        <v>E</v>
+      </c>
+      <c r="K34" t="str">
+        <v>E</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
         <v>C9</v>
       </c>
-      <c r="N33" t="str">
-        <v>E</v>
-      </c>
-      <c r="O33" t="str">
-        <v/>
-      </c>
-      <c r="P33" t="str">
+      <c r="N34" t="str">
+        <v>E</v>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+      <c r="P34" t="str">
         <v>C9</v>
       </c>
-      <c r="Q33" t="str">
-        <v/>
-      </c>
-      <c r="R33" t="str">
-        <v/>
-      </c>
-      <c r="S33" t="str">
-        <v/>
-      </c>
-      <c r="T33" t="str">
-        <v/>
-      </c>
-      <c r="U33" t="str">
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
         <v>C9</v>
       </c>
-      <c r="V33" t="str">
-        <v/>
-      </c>
-      <c r="W33" t="str">
-        <v>M</v>
-      </c>
-      <c r="X33" t="str">
+      <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
+        <v>M</v>
+      </c>
+      <c r="X34" t="str">
         <v>C9</v>
       </c>
-      <c r="Y33" t="str">
-        <v/>
-      </c>
-      <c r="Z33" t="str">
+      <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
         <v>C9</v>
       </c>
-      <c r="AA33" t="str">
+      <c r="AA34" t="str">
         <v>C9</v>
       </c>
-      <c r="AB33" t="str">
-        <v>E</v>
-      </c>
-      <c r="AC33" t="str">
-        <v/>
-      </c>
-      <c r="AD33" t="str">
+      <c r="AB34" t="str">
+        <v>E</v>
+      </c>
+      <c r="AC34" t="str">
+        <v/>
+      </c>
+      <c r="AD34" t="str">
         <v>C9</v>
       </c>
-      <c r="AE33" t="str">
-        <v/>
-      </c>
-      <c r="AF33" t="str">
-        <v/>
-      </c>
-      <c r="AG33" t="str">
-        <v>E</v>
-      </c>
-      <c r="AH33" t="str">
+      <c r="AE34" t="str">
+        <v/>
+      </c>
+      <c r="AF34" t="str">
+        <v/>
+      </c>
+      <c r="AG34" t="str">
+        <v>E</v>
+      </c>
+      <c r="AH34" t="str">
         <v>C9</v>
       </c>
-      <c r="AI33">
-        <v>0</v>
-      </c>
-      <c r="AJ33">
+      <c r="AI34">
+        <v>0</v>
+      </c>
+      <c r="AJ34">
         <v>2</v>
       </c>
-      <c r="AK33">
+      <c r="AK34">
         <v>6</v>
       </c>
-      <c r="AL33">
+      <c r="AL34">
         <v>10</v>
       </c>
-      <c r="AM33">
-        <v>0</v>
-      </c>
-      <c r="AN33">
+      <c r="AM34">
+        <v>0</v>
+      </c>
+      <c r="AN34">
         <v>216</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 09/2026 from web (21 NV)
</commit_message>
<xml_diff>
--- a/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
+++ b/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN33"/>
+  <dimension ref="A1:AN32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1401,19 +1401,19 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v>DSP HDQ</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>30904</v>
       </c>
       <c r="C18" t="str">
-        <v>Nguyễn Phương Linh</v>
+        <v>Trần Đình Đạt</v>
       </c>
       <c r="D18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -1425,31 +1425,31 @@
         <v/>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="K18" t="str">
-        <v/>
+        <v>NL</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O18" t="str">
         <v/>
       </c>
       <c r="P18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R18" t="str">
         <v/>
@@ -1458,22 +1458,22 @@
         <v/>
       </c>
       <c r="T18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V18" t="str">
         <v/>
       </c>
       <c r="W18" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="X18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z18" t="str">
         <v/>
@@ -1482,10 +1482,10 @@
         <v/>
       </c>
       <c r="AB18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD18" t="str">
         <v/>
@@ -1494,48 +1494,48 @@
         <v/>
       </c>
       <c r="AF18" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AG18" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH18" t="str">
         <v/>
       </c>
       <c r="AI18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ18">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AK18">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AL18">
         <v>0</v>
       </c>
       <c r="AM18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN18">
-        <v>0</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>DSP HDQ</v>
+        <v/>
       </c>
       <c r="B19" t="str">
-        <v>30904</v>
+        <v>30905</v>
       </c>
       <c r="C19" t="str">
-        <v>Trần Đình Đạt</v>
+        <v>Nguyễn Trương Hoàng Hưng</v>
       </c>
       <c r="D19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="E19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -1544,94 +1544,94 @@
         <v/>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="J19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="K19" t="str">
         <v>NL</v>
       </c>
       <c r="L19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M19" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="N19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O19" t="str">
         <v/>
       </c>
       <c r="P19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V19" t="str">
         <v/>
       </c>
       <c r="W19" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="X19" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA19" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AC19" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE19" t="str">
         <v/>
       </c>
       <c r="AF19" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG19" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AH19" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AI19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ19">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AK19">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AL19">
         <v>0</v>
@@ -1640,7 +1640,7 @@
         <v>1</v>
       </c>
       <c r="AN19">
-        <v>220</v>
+        <v>212</v>
       </c>
     </row>
     <row r="20">
@@ -1648,46 +1648,46 @@
         <v/>
       </c>
       <c r="B20" t="str">
-        <v>30905</v>
+        <v>30841</v>
       </c>
       <c r="C20" t="str">
-        <v>Nguyễn Trương Hoàng Hưng</v>
+        <v>Vũ Hoàng Long</v>
       </c>
       <c r="D20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="H20" t="str">
-        <v>M</v>
+        <v>P</v>
       </c>
       <c r="I20" t="str">
-        <v>E</v>
+        <v>P</v>
       </c>
       <c r="J20" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="K20" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L20" t="str">
         <v/>
       </c>
       <c r="M20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="P20" t="str">
         <v>E</v>
@@ -1699,22 +1699,22 @@
         <v>M</v>
       </c>
       <c r="S20" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="T20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U20" t="str">
         <v/>
       </c>
       <c r="V20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W20" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y20" t="str">
         <v/>
@@ -1723,37 +1723,37 @@
         <v>M</v>
       </c>
       <c r="AA20" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AB20" t="str">
         <v/>
       </c>
       <c r="AC20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD20" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE20" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AF20" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG20" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AH20" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AI20">
         <v>0</v>
       </c>
       <c r="AJ20">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AK20">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AL20">
         <v>0</v>
@@ -1762,7 +1762,7 @@
         <v>1</v>
       </c>
       <c r="AN20">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="21">
@@ -1770,97 +1770,97 @@
         <v/>
       </c>
       <c r="B21" t="str">
-        <v>30841</v>
+        <v>29718</v>
       </c>
       <c r="C21" t="str">
-        <v>Vũ Hoàng Long</v>
+        <v>Vũ Huy Hùng</v>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>HC</v>
       </c>
       <c r="F21" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="G21" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="H21" t="str">
-        <v>P</v>
+        <v/>
       </c>
       <c r="I21" t="str">
-        <v>P</v>
+        <v>HC</v>
       </c>
       <c r="J21" t="str">
+        <v>M</v>
+      </c>
+      <c r="K21" t="str">
         <v>NL</v>
       </c>
-      <c r="K21" t="str">
-        <v>E</v>
-      </c>
       <c r="L21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="O21" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="P21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T21" t="str">
         <v/>
       </c>
       <c r="U21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="V21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X21" t="str">
         <v/>
       </c>
       <c r="Y21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Z21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AA21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB21" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC21" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD21" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE21" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AF21" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AG21" t="str">
         <v/>
@@ -1869,10 +1869,10 @@
         <v>M</v>
       </c>
       <c r="AI21">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AJ21">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AK21">
         <v>7</v>
@@ -1889,49 +1889,49 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>DSP ASST HDQ</v>
       </c>
       <c r="B22" t="str">
-        <v>29718</v>
+        <v>39278</v>
       </c>
       <c r="C22" t="str">
-        <v>Vũ Huy Hùng</v>
+        <v>Nguyền Kiều Huyền Chi</v>
       </c>
       <c r="D22" t="str">
-        <v>HC</v>
+        <v>E</v>
       </c>
       <c r="E22" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="F22" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="G22" t="str">
-        <v>HC</v>
+        <v>M</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I22" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="J22" t="str">
         <v>M</v>
       </c>
       <c r="K22" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="L22" t="str">
         <v>E</v>
       </c>
       <c r="M22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="O22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P22" t="str">
         <v/>
@@ -1940,10 +1940,10 @@
         <v>M</v>
       </c>
       <c r="R22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="S22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="T22" t="str">
         <v/>
@@ -1955,165 +1955,165 @@
         <v>E</v>
       </c>
       <c r="W22" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="X22" t="str">
         <v/>
       </c>
       <c r="Y22" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Z22" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AA22" t="str">
         <v/>
       </c>
       <c r="AB22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC22" t="str">
         <v/>
       </c>
       <c r="AD22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AE22" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AF22" t="str">
-        <v/>
+        <v>C349</v>
       </c>
       <c r="AG22" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AH22" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AI22">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AJ22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AK22">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AL22">
         <v>0</v>
       </c>
       <c r="AM22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN22">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>DSP ASST HDQ</v>
+        <v/>
       </c>
       <c r="B23" t="str">
-        <v>39278</v>
+        <v>39280</v>
       </c>
       <c r="C23" t="str">
-        <v>Nguyền Kiều Huyền Chi</v>
+        <v>Đặng Thảo Linh</v>
       </c>
       <c r="D23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E23" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="G23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="H23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="I23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J23" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="K23" t="str">
         <v>M</v>
       </c>
       <c r="L23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="M23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="N23" t="str">
-        <v>SN</v>
+        <v/>
       </c>
       <c r="O23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="P23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Q23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="R23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="S23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="T23" t="str">
         <v/>
       </c>
       <c r="U23" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W23" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="X23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y23" t="str">
         <v/>
       </c>
       <c r="Z23" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="AA23" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC23" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD23" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AE23" t="str">
         <v/>
       </c>
       <c r="AF23" t="str">
-        <v>C349</v>
+        <v>M</v>
       </c>
       <c r="AG23" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AH23" t="str">
         <v>E</v>
       </c>
       <c r="AI23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ23">
         <v>8</v>
@@ -2125,10 +2125,10 @@
         <v>0</v>
       </c>
       <c r="AM23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN23">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24">
@@ -2136,64 +2136,64 @@
         <v/>
       </c>
       <c r="B24" t="str">
-        <v>39280</v>
+        <v>39276</v>
       </c>
       <c r="C24" t="str">
-        <v>Đặng Thảo Linh</v>
+        <v>Bùi Việt Anh</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="E24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="I24" t="str">
         <v>E</v>
       </c>
       <c r="J24" t="str">
+        <v>E</v>
+      </c>
+      <c r="K24" t="str">
         <v>NL</v>
       </c>
-      <c r="K24" t="str">
-        <v>M</v>
-      </c>
       <c r="L24" t="str">
-        <v>M</v>
+        <v>P</v>
       </c>
       <c r="M24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="O24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="P24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="R24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="U24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V24" t="str">
         <v/>
@@ -2202,46 +2202,46 @@
         <v>M</v>
       </c>
       <c r="X24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="Z24" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AA24" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AB24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AD24" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE24" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF24" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG24" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AH24" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AI24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ24">
+        <v>9</v>
+      </c>
+      <c r="AK24">
         <v>8</v>
-      </c>
-      <c r="AK24">
-        <v>9</v>
       </c>
       <c r="AL24">
         <v>0</v>
@@ -2258,19 +2258,19 @@
         <v/>
       </c>
       <c r="B25" t="str">
-        <v>39276</v>
+        <v>39274</v>
       </c>
       <c r="C25" t="str">
-        <v>Bùi Việt Anh</v>
+        <v>Đỗ Nam Anh</v>
       </c>
       <c r="D25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="E25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G25" t="str">
         <v/>
@@ -2279,82 +2279,82 @@
         <v>M</v>
       </c>
       <c r="I25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="J25" t="str">
         <v>E</v>
       </c>
       <c r="K25" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L25" t="str">
-        <v>P</v>
+        <v/>
       </c>
       <c r="M25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="N25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O25" t="str">
         <v/>
       </c>
       <c r="P25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R25" t="str">
         <v/>
       </c>
       <c r="S25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="T25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="W25" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="X25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Y25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="Z25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AA25" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AB25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AC25" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AD25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE25" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="AF25" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AG25" t="str">
         <v/>
       </c>
       <c r="AH25" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AI25">
         <v>0</v>
@@ -2363,87 +2363,87 @@
         <v>9</v>
       </c>
       <c r="AK25">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AL25">
         <v>0</v>
       </c>
       <c r="AM25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN25">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v/>
+        <v>DSP SGN</v>
       </c>
       <c r="B26" t="str">
-        <v>39274</v>
+        <v>31844</v>
       </c>
       <c r="C26" t="str">
-        <v>Đỗ Nam Anh</v>
+        <v>Nguyễn Hoàng Huy</v>
       </c>
       <c r="D26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="E26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="F26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>SN</v>
       </c>
       <c r="H26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="J26" t="str">
         <v>E</v>
       </c>
       <c r="K26" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="L26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="M26" t="str">
         <v>M</v>
       </c>
       <c r="N26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="O26" t="str">
         <v/>
       </c>
       <c r="P26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="R26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="S26" t="str">
         <v/>
       </c>
       <c r="T26" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="U26" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="W26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X26" t="str">
         <v/>
@@ -2452,22 +2452,22 @@
         <v>M</v>
       </c>
       <c r="Z26" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AA26" t="str">
         <v/>
       </c>
       <c r="AB26" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AC26" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AE26" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="AF26" t="str">
         <v>E</v>
@@ -2476,22 +2476,22 @@
         <v/>
       </c>
       <c r="AH26" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AI26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ26">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AK26">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AL26">
         <v>0</v>
       </c>
       <c r="AM26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN26">
         <v>216</v>
@@ -2499,106 +2499,106 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>DSP SGN</v>
+        <v/>
       </c>
       <c r="B27" t="str">
-        <v>31844</v>
+        <v>31843</v>
       </c>
       <c r="C27" t="str">
-        <v>Nguyễn Hoàng Huy</v>
+        <v>Lương Trung Hiếu</v>
       </c>
       <c r="D27" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="G27" t="str">
-        <v>SN</v>
+        <v>E</v>
       </c>
       <c r="H27" t="str">
         <v/>
       </c>
       <c r="I27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="J27" t="str">
-        <v>E</v>
+        <v>NL</v>
       </c>
       <c r="K27" t="str">
         <v>NL</v>
       </c>
       <c r="L27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="M27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="O27" t="str">
         <v/>
       </c>
       <c r="P27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="R27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="S27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="T27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="U27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="V27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="W27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="X27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y27" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Z27" t="str">
         <v/>
       </c>
       <c r="AA27" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AB27" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="AC27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AD27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AE27" t="str">
+        <v>M</v>
+      </c>
+      <c r="AF27" t="str">
         <v>HC</v>
       </c>
-      <c r="AF27" t="str">
-        <v>E</v>
-      </c>
       <c r="AG27" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AH27" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AI27">
         <v>1</v>
@@ -2613,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="AM27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN27">
         <v>216</v>
@@ -2624,61 +2624,61 @@
         <v/>
       </c>
       <c r="B28" t="str">
-        <v>31843</v>
+        <v>31846</v>
       </c>
       <c r="C28" t="str">
-        <v>Lương Trung Hiếu</v>
+        <v>Nguyễn Phúc Thịnh</v>
       </c>
       <c r="D28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="E28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F28" t="str">
         <v/>
       </c>
       <c r="G28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="H28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="I28" t="str">
         <v/>
       </c>
       <c r="J28" t="str">
-        <v>NL</v>
+        <v>M</v>
       </c>
       <c r="K28" t="str">
-        <v>NL</v>
+        <v>E</v>
       </c>
       <c r="L28" t="str">
         <v/>
       </c>
       <c r="M28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="N28" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="P28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Q28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="R28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="S28" t="str">
-        <v>M</v>
+        <v>HC</v>
       </c>
       <c r="T28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="U28" t="str">
         <v/>
@@ -2687,19 +2687,19 @@
         <v/>
       </c>
       <c r="W28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="X28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y28" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Z28" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="AA28" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="AB28" t="str">
         <v/>
@@ -2708,37 +2708,37 @@
         <v>E</v>
       </c>
       <c r="AD28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AE28" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AF28" t="str">
+        <v>M</v>
+      </c>
+      <c r="AG28" t="str">
         <v>HC</v>
       </c>
-      <c r="AG28" t="str">
-        <v>E</v>
-      </c>
       <c r="AH28" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AI28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AJ28">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK28">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AL28">
         <v>0</v>
       </c>
       <c r="AM28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AN28">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29">
@@ -2746,153 +2746,153 @@
         <v/>
       </c>
       <c r="B29" t="str">
-        <v>31846</v>
+        <v>31847</v>
       </c>
       <c r="C29" t="str">
-        <v>Nguyễn Phúc Thịnh</v>
+        <v>Hoàng Bảo Ngọc</v>
       </c>
       <c r="D29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="E29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="G29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="H29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="I29" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="J29" t="str">
-        <v>M</v>
+        <v>NL</v>
       </c>
       <c r="K29" t="str">
-        <v>E</v>
+        <v>M</v>
       </c>
       <c r="L29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="M29" t="str">
         <v/>
       </c>
       <c r="N29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="O29" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="P29" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="Q29" t="str">
         <v/>
       </c>
       <c r="R29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="S29" t="str">
+        <v>E</v>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v>M</v>
+      </c>
+      <c r="V29" t="str">
+        <v>M</v>
+      </c>
+      <c r="W29" t="str">
+        <v>E</v>
+      </c>
+      <c r="X29" t="str">
+        <v/>
+      </c>
+      <c r="Y29" t="str">
+        <v/>
+      </c>
+      <c r="Z29" t="str">
+        <v>E</v>
+      </c>
+      <c r="AA29" t="str">
+        <v/>
+      </c>
+      <c r="AB29" t="str">
+        <v>M</v>
+      </c>
+      <c r="AC29" t="str">
+        <v>M</v>
+      </c>
+      <c r="AD29" t="str">
         <v>HC</v>
       </c>
-      <c r="T29" t="str">
-        <v/>
-      </c>
-      <c r="U29" t="str">
-        <v/>
-      </c>
-      <c r="V29" t="str">
-        <v/>
-      </c>
-      <c r="W29" t="str">
-        <v/>
-      </c>
-      <c r="X29" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y29" t="str">
-        <v/>
-      </c>
-      <c r="Z29" t="str">
-        <v>M</v>
-      </c>
-      <c r="AA29" t="str">
-        <v>E</v>
-      </c>
-      <c r="AB29" t="str">
-        <v/>
-      </c>
-      <c r="AC29" t="str">
-        <v>E</v>
-      </c>
-      <c r="AD29" t="str">
-        <v>E</v>
-      </c>
       <c r="AE29" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AF29" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AG29" t="str">
+        <v>M</v>
+      </c>
+      <c r="AH29" t="str">
         <v>HC</v>
-      </c>
-      <c r="AH29" t="str">
-        <v>E</v>
       </c>
       <c r="AI29">
         <v>2</v>
       </c>
       <c r="AJ29">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AK29">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AL29">
         <v>0</v>
       </c>
       <c r="AM29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN29">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v/>
+        <v>DSP PQC</v>
       </c>
       <c r="B30" t="str">
-        <v>31847</v>
+        <v>41863</v>
       </c>
       <c r="C30" t="str">
-        <v>Hoàng Bảo Ngọc</v>
+        <v>Lê Ngọc Thành Tài</v>
       </c>
       <c r="D30" t="str">
         <v/>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="F30" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="G30" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="H30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="I30" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="J30" t="str">
-        <v>NL</v>
+        <v>C9</v>
       </c>
       <c r="K30" t="str">
         <v>M</v>
@@ -2904,40 +2904,40 @@
         <v/>
       </c>
       <c r="N30" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="O30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="P30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Q30" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="R30" t="str">
         <v/>
       </c>
       <c r="S30" t="str">
-        <v>E</v>
+        <v>C9</v>
       </c>
       <c r="T30" t="str">
         <v/>
       </c>
       <c r="U30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="V30" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="W30" t="str">
-        <v>E</v>
+        <v/>
       </c>
       <c r="X30" t="str">
-        <v/>
+        <v>M</v>
       </c>
       <c r="Y30" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="Z30" t="str">
         <v>E</v>
@@ -2946,13 +2946,13 @@
         <v/>
       </c>
       <c r="AB30" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="AC30" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="AD30" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AE30" t="str">
         <v>E</v>
@@ -2961,25 +2961,25 @@
         <v/>
       </c>
       <c r="AG30" t="str">
-        <v>M</v>
+        <v>C9</v>
       </c>
       <c r="AH30" t="str">
-        <v>HC</v>
+        <v/>
       </c>
       <c r="AI30">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ30">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AK30">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AL30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AM30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN30">
         <v>216</v>
@@ -2987,103 +2987,103 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>DSP PQC</v>
+        <v/>
       </c>
       <c r="B31" t="str">
-        <v>41863</v>
+        <v>41865</v>
       </c>
       <c r="C31" t="str">
-        <v>Lê Ngọc Thành Tài</v>
+        <v>Nguyễn Đức Lộc</v>
       </c>
       <c r="D31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="E31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="F31" t="str">
+        <v/>
+      </c>
+      <c r="G31" t="str">
         <v>C9</v>
       </c>
-      <c r="G31" t="str">
-        <v>E</v>
-      </c>
       <c r="H31" t="str">
         <v/>
       </c>
       <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v>M</v>
+      </c>
+      <c r="K31" t="str">
         <v>C9</v>
       </c>
-      <c r="J31" t="str">
+      <c r="L31" t="str">
         <v>C9</v>
       </c>
-      <c r="K31" t="str">
-        <v>M</v>
-      </c>
-      <c r="L31" t="str">
-        <v>E</v>
-      </c>
       <c r="M31" t="str">
         <v/>
       </c>
       <c r="N31" t="str">
+        <v/>
+      </c>
+      <c r="O31" t="str">
         <v>C9</v>
       </c>
-      <c r="O31" t="str">
-        <v/>
-      </c>
       <c r="P31" t="str">
-        <v>M</v>
+        <v/>
       </c>
       <c r="Q31" t="str">
+        <v>M</v>
+      </c>
+      <c r="R31" t="str">
         <v>C9</v>
       </c>
-      <c r="R31" t="str">
-        <v/>
-      </c>
       <c r="S31" t="str">
+        <v/>
+      </c>
+      <c r="T31" t="str">
         <v>C9</v>
       </c>
-      <c r="T31" t="str">
-        <v/>
-      </c>
       <c r="U31" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="V31" t="str">
+        <v/>
+      </c>
+      <c r="W31" t="str">
         <v>C9</v>
       </c>
-      <c r="W31" t="str">
-        <v/>
-      </c>
       <c r="X31" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="Y31" t="str">
+        <v/>
+      </c>
+      <c r="Z31" t="str">
+        <v>M</v>
+      </c>
+      <c r="AA31" t="str">
+        <v/>
+      </c>
+      <c r="AB31" t="str">
+        <v/>
+      </c>
+      <c r="AC31" t="str">
         <v>C9</v>
       </c>
-      <c r="Z31" t="str">
-        <v>E</v>
-      </c>
-      <c r="AA31" t="str">
-        <v/>
-      </c>
-      <c r="AB31" t="str">
+      <c r="AD31" t="str">
+        <v/>
+      </c>
+      <c r="AE31" t="str">
         <v>C9</v>
       </c>
-      <c r="AC31" t="str">
-        <v/>
-      </c>
-      <c r="AD31" t="str">
-        <v/>
-      </c>
-      <c r="AE31" t="str">
-        <v>E</v>
-      </c>
       <c r="AF31" t="str">
-        <v/>
+        <v>C9</v>
       </c>
       <c r="AG31" t="str">
-        <v>C9</v>
+        <v>M</v>
       </c>
       <c r="AH31" t="str">
         <v/>
@@ -3095,10 +3095,10 @@
         <v>4</v>
       </c>
       <c r="AK31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AL31">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="AM31">
         <v>0</v>
@@ -3112,248 +3112,126 @@
         <v/>
       </c>
       <c r="B32" t="str">
-        <v>41865</v>
+        <v>41867</v>
       </c>
       <c r="C32" t="str">
-        <v>Nguyễn Đức Lộc</v>
+        <v>Phan Thành Nghĩa</v>
       </c>
       <c r="D32" t="str">
+        <v>M</v>
+      </c>
+      <c r="E32" t="str">
         <v>C9</v>
       </c>
-      <c r="E32" t="str">
-        <v>E</v>
-      </c>
       <c r="F32" t="str">
         <v/>
       </c>
       <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
         <v>C9</v>
       </c>
-      <c r="H32" t="str">
-        <v/>
-      </c>
       <c r="I32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="J32" t="str">
-        <v>M</v>
+        <v>E</v>
       </c>
       <c r="K32" t="str">
+        <v>E</v>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
         <v>C9</v>
       </c>
-      <c r="L32" t="str">
+      <c r="N32" t="str">
+        <v>E</v>
+      </c>
+      <c r="O32" t="str">
+        <v/>
+      </c>
+      <c r="P32" t="str">
         <v>C9</v>
       </c>
-      <c r="M32" t="str">
-        <v/>
-      </c>
-      <c r="N32" t="str">
-        <v/>
-      </c>
-      <c r="O32" t="str">
+      <c r="Q32" t="str">
+        <v/>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
+        <v/>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
         <v>C9</v>
       </c>
-      <c r="P32" t="str">
-        <v/>
-      </c>
-      <c r="Q32" t="str">
-        <v>M</v>
-      </c>
-      <c r="R32" t="str">
+      <c r="V32" t="str">
+        <v/>
+      </c>
+      <c r="W32" t="str">
+        <v>M</v>
+      </c>
+      <c r="X32" t="str">
         <v>C9</v>
       </c>
-      <c r="S32" t="str">
-        <v/>
-      </c>
-      <c r="T32" t="str">
+      <c r="Y32" t="str">
+        <v/>
+      </c>
+      <c r="Z32" t="str">
         <v>C9</v>
       </c>
-      <c r="U32" t="str">
-        <v>E</v>
-      </c>
-      <c r="V32" t="str">
-        <v/>
-      </c>
-      <c r="W32" t="str">
+      <c r="AA32" t="str">
         <v>C9</v>
       </c>
-      <c r="X32" t="str">
-        <v>E</v>
-      </c>
-      <c r="Y32" t="str">
-        <v/>
-      </c>
-      <c r="Z32" t="str">
-        <v>M</v>
-      </c>
-      <c r="AA32" t="str">
-        <v/>
-      </c>
       <c r="AB32" t="str">
-        <v/>
+        <v>E</v>
       </c>
       <c r="AC32" t="str">
+        <v/>
+      </c>
+      <c r="AD32" t="str">
         <v>C9</v>
       </c>
-      <c r="AD32" t="str">
-        <v/>
-      </c>
       <c r="AE32" t="str">
+        <v/>
+      </c>
+      <c r="AF32" t="str">
+        <v/>
+      </c>
+      <c r="AG32" t="str">
+        <v>E</v>
+      </c>
+      <c r="AH32" t="str">
         <v>C9</v>
       </c>
-      <c r="AF32" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AG32" t="str">
-        <v>M</v>
-      </c>
-      <c r="AH32" t="str">
-        <v/>
-      </c>
       <c r="AI32">
         <v>0</v>
       </c>
       <c r="AJ32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AK32">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="AL32">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AM32">
         <v>0</v>
       </c>
       <c r="AN32">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v/>
-      </c>
-      <c r="B33" t="str">
-        <v>41867</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Phan Thành Nghĩa</v>
-      </c>
-      <c r="D33" t="str">
-        <v>M</v>
-      </c>
-      <c r="E33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="F33" t="str">
-        <v/>
-      </c>
-      <c r="G33" t="str">
-        <v/>
-      </c>
-      <c r="H33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="I33" t="str">
-        <v>E</v>
-      </c>
-      <c r="J33" t="str">
-        <v>E</v>
-      </c>
-      <c r="K33" t="str">
-        <v>E</v>
-      </c>
-      <c r="L33" t="str">
-        <v/>
-      </c>
-      <c r="M33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="N33" t="str">
-        <v>E</v>
-      </c>
-      <c r="O33" t="str">
-        <v/>
-      </c>
-      <c r="P33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="Q33" t="str">
-        <v/>
-      </c>
-      <c r="R33" t="str">
-        <v/>
-      </c>
-      <c r="S33" t="str">
-        <v/>
-      </c>
-      <c r="T33" t="str">
-        <v/>
-      </c>
-      <c r="U33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="V33" t="str">
-        <v/>
-      </c>
-      <c r="W33" t="str">
-        <v>M</v>
-      </c>
-      <c r="X33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="Y33" t="str">
-        <v/>
-      </c>
-      <c r="Z33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AA33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AB33" t="str">
-        <v>E</v>
-      </c>
-      <c r="AC33" t="str">
-        <v/>
-      </c>
-      <c r="AD33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AE33" t="str">
-        <v/>
-      </c>
-      <c r="AF33" t="str">
-        <v/>
-      </c>
-      <c r="AG33" t="str">
-        <v>E</v>
-      </c>
-      <c r="AH33" t="str">
-        <v>C9</v>
-      </c>
-      <c r="AI33">
-        <v>0</v>
-      </c>
-      <c r="AJ33">
-        <v>2</v>
-      </c>
-      <c r="AK33">
-        <v>6</v>
-      </c>
-      <c r="AL33">
-        <v>10</v>
-      </c>
-      <c r="AM33">
-        <v>0</v>
-      </c>
-      <c r="AN33">
         <v>216</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 09/2026 from web (25 NV)
</commit_message>
<xml_diff>
--- a/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
+++ b/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN32"/>
+  <dimension ref="A1:AN36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3229,9 +3229,497 @@
         <v>216</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Briefing PQC</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33" t="str">
+        <v>Phan Như Ngọc</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v/>
+      </c>
+      <c r="AA33" t="str">
+        <v/>
+      </c>
+      <c r="AB33" t="str">
+        <v/>
+      </c>
+      <c r="AC33" t="str">
+        <v/>
+      </c>
+      <c r="AD33" t="str">
+        <v/>
+      </c>
+      <c r="AE33" t="str">
+        <v/>
+      </c>
+      <c r="AF33" t="str">
+        <v/>
+      </c>
+      <c r="AG33" t="str">
+        <v/>
+      </c>
+      <c r="AH33" t="str">
+        <v/>
+      </c>
+      <c r="AI33">
+        <v>0</v>
+      </c>
+      <c r="AJ33">
+        <v>0</v>
+      </c>
+      <c r="AK33">
+        <v>0</v>
+      </c>
+      <c r="AL33">
+        <v>0</v>
+      </c>
+      <c r="AM33">
+        <v>0</v>
+      </c>
+      <c r="AN33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v>Phan Hiền Phúc Đạt</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v/>
+      </c>
+      <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
+        <v/>
+      </c>
+      <c r="X34" t="str">
+        <v/>
+      </c>
+      <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
+        <v/>
+      </c>
+      <c r="AA34" t="str">
+        <v/>
+      </c>
+      <c r="AB34" t="str">
+        <v/>
+      </c>
+      <c r="AC34" t="str">
+        <v/>
+      </c>
+      <c r="AD34" t="str">
+        <v/>
+      </c>
+      <c r="AE34" t="str">
+        <v/>
+      </c>
+      <c r="AF34" t="str">
+        <v/>
+      </c>
+      <c r="AG34" t="str">
+        <v/>
+      </c>
+      <c r="AH34" t="str">
+        <v/>
+      </c>
+      <c r="AI34">
+        <v>0</v>
+      </c>
+      <c r="AJ34">
+        <v>0</v>
+      </c>
+      <c r="AK34">
+        <v>0</v>
+      </c>
+      <c r="AL34">
+        <v>0</v>
+      </c>
+      <c r="AM34">
+        <v>0</v>
+      </c>
+      <c r="AN34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v>Nguyễn Phạm Quỳnh Trang</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
+        <v/>
+      </c>
+      <c r="V35" t="str">
+        <v/>
+      </c>
+      <c r="W35" t="str">
+        <v/>
+      </c>
+      <c r="X35" t="str">
+        <v/>
+      </c>
+      <c r="Y35" t="str">
+        <v/>
+      </c>
+      <c r="Z35" t="str">
+        <v/>
+      </c>
+      <c r="AA35" t="str">
+        <v/>
+      </c>
+      <c r="AB35" t="str">
+        <v/>
+      </c>
+      <c r="AC35" t="str">
+        <v/>
+      </c>
+      <c r="AD35" t="str">
+        <v/>
+      </c>
+      <c r="AE35" t="str">
+        <v/>
+      </c>
+      <c r="AF35" t="str">
+        <v/>
+      </c>
+      <c r="AG35" t="str">
+        <v/>
+      </c>
+      <c r="AH35" t="str">
+        <v/>
+      </c>
+      <c r="AI35">
+        <v>0</v>
+      </c>
+      <c r="AJ35">
+        <v>0</v>
+      </c>
+      <c r="AK35">
+        <v>0</v>
+      </c>
+      <c r="AL35">
+        <v>0</v>
+      </c>
+      <c r="AM35">
+        <v>0</v>
+      </c>
+      <c r="AN35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v>Nguyễn Phương Linh</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
+        <v/>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v/>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
+      <c r="W36" t="str">
+        <v/>
+      </c>
+      <c r="X36" t="str">
+        <v/>
+      </c>
+      <c r="Y36" t="str">
+        <v/>
+      </c>
+      <c r="Z36" t="str">
+        <v/>
+      </c>
+      <c r="AA36" t="str">
+        <v/>
+      </c>
+      <c r="AB36" t="str">
+        <v/>
+      </c>
+      <c r="AC36" t="str">
+        <v/>
+      </c>
+      <c r="AD36" t="str">
+        <v/>
+      </c>
+      <c r="AE36" t="str">
+        <v/>
+      </c>
+      <c r="AF36" t="str">
+        <v/>
+      </c>
+      <c r="AG36" t="str">
+        <v/>
+      </c>
+      <c r="AH36" t="str">
+        <v/>
+      </c>
+      <c r="AI36">
+        <v>0</v>
+      </c>
+      <c r="AJ36">
+        <v>0</v>
+      </c>
+      <c r="AK36">
+        <v>0</v>
+      </c>
+      <c r="AL36">
+        <v>0</v>
+      </c>
+      <c r="AM36">
+        <v>0</v>
+      </c>
+      <c r="AN36">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update roster 09/2026 from web (29 NV)
</commit_message>
<xml_diff>
--- a/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
+++ b/data/2026/09.2026/Lịch trực OCD on SEP final 15Sep26 (2).xlsx
@@ -32,12 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -401,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN32"/>
+  <dimension ref="A1:AN40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3233,9 +3229,985 @@
         <v>216</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>BRF SGN</v>
+      </c>
+      <c r="B33" t="str">
+        <v>32117</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Lê Song Huyền Vi</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+      <c r="F33" t="str">
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v/>
+      </c>
+      <c r="AA33" t="str">
+        <v/>
+      </c>
+      <c r="AB33" t="str">
+        <v/>
+      </c>
+      <c r="AC33" t="str">
+        <v/>
+      </c>
+      <c r="AD33" t="str">
+        <v/>
+      </c>
+      <c r="AE33" t="str">
+        <v/>
+      </c>
+      <c r="AF33" t="str">
+        <v/>
+      </c>
+      <c r="AG33" t="str">
+        <v/>
+      </c>
+      <c r="AH33" t="str">
+        <v/>
+      </c>
+      <c r="AI33">
+        <v>0</v>
+      </c>
+      <c r="AJ33">
+        <v>0</v>
+      </c>
+      <c r="AK33">
+        <v>0</v>
+      </c>
+      <c r="AL33">
+        <v>0</v>
+      </c>
+      <c r="AM33">
+        <v>0</v>
+      </c>
+      <c r="AN33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v>32115</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Đoàn Văn Tây</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v/>
+      </c>
+      <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
+        <v/>
+      </c>
+      <c r="X34" t="str">
+        <v/>
+      </c>
+      <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
+        <v/>
+      </c>
+      <c r="AA34" t="str">
+        <v/>
+      </c>
+      <c r="AB34" t="str">
+        <v/>
+      </c>
+      <c r="AC34" t="str">
+        <v/>
+      </c>
+      <c r="AD34" t="str">
+        <v/>
+      </c>
+      <c r="AE34" t="str">
+        <v/>
+      </c>
+      <c r="AF34" t="str">
+        <v/>
+      </c>
+      <c r="AG34" t="str">
+        <v/>
+      </c>
+      <c r="AH34" t="str">
+        <v/>
+      </c>
+      <c r="AI34">
+        <v>0</v>
+      </c>
+      <c r="AJ34">
+        <v>0</v>
+      </c>
+      <c r="AK34">
+        <v>0</v>
+      </c>
+      <c r="AL34">
+        <v>0</v>
+      </c>
+      <c r="AM34">
+        <v>0</v>
+      </c>
+      <c r="AN34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v>31969</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Nguyễn Thị Mỹ Hương</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v/>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v/>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
+        <v/>
+      </c>
+      <c r="V35" t="str">
+        <v/>
+      </c>
+      <c r="W35" t="str">
+        <v/>
+      </c>
+      <c r="X35" t="str">
+        <v/>
+      </c>
+      <c r="Y35" t="str">
+        <v/>
+      </c>
+      <c r="Z35" t="str">
+        <v/>
+      </c>
+      <c r="AA35" t="str">
+        <v/>
+      </c>
+      <c r="AB35" t="str">
+        <v/>
+      </c>
+      <c r="AC35" t="str">
+        <v/>
+      </c>
+      <c r="AD35" t="str">
+        <v/>
+      </c>
+      <c r="AE35" t="str">
+        <v/>
+      </c>
+      <c r="AF35" t="str">
+        <v/>
+      </c>
+      <c r="AG35" t="str">
+        <v/>
+      </c>
+      <c r="AH35" t="str">
+        <v/>
+      </c>
+      <c r="AI35">
+        <v>0</v>
+      </c>
+      <c r="AJ35">
+        <v>0</v>
+      </c>
+      <c r="AK35">
+        <v>0</v>
+      </c>
+      <c r="AL35">
+        <v>0</v>
+      </c>
+      <c r="AM35">
+        <v>0</v>
+      </c>
+      <c r="AN35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v>37388</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Trương Thị Ngọc Loan</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v/>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
+        <v/>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v/>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
+      <c r="W36" t="str">
+        <v/>
+      </c>
+      <c r="X36" t="str">
+        <v/>
+      </c>
+      <c r="Y36" t="str">
+        <v/>
+      </c>
+      <c r="Z36" t="str">
+        <v/>
+      </c>
+      <c r="AA36" t="str">
+        <v/>
+      </c>
+      <c r="AB36" t="str">
+        <v/>
+      </c>
+      <c r="AC36" t="str">
+        <v/>
+      </c>
+      <c r="AD36" t="str">
+        <v/>
+      </c>
+      <c r="AE36" t="str">
+        <v/>
+      </c>
+      <c r="AF36" t="str">
+        <v/>
+      </c>
+      <c r="AG36" t="str">
+        <v/>
+      </c>
+      <c r="AH36" t="str">
+        <v/>
+      </c>
+      <c r="AI36">
+        <v>0</v>
+      </c>
+      <c r="AJ36">
+        <v>0</v>
+      </c>
+      <c r="AK36">
+        <v>0</v>
+      </c>
+      <c r="AL36">
+        <v>0</v>
+      </c>
+      <c r="AM36">
+        <v>0</v>
+      </c>
+      <c r="AN36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>BRF PQC</v>
+      </c>
+      <c r="B37" t="str">
+        <v>41366</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Phan Như Ngọc</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v/>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v/>
+      </c>
+      <c r="N37" t="str">
+        <v/>
+      </c>
+      <c r="O37" t="str">
+        <v/>
+      </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
+      <c r="R37" t="str">
+        <v/>
+      </c>
+      <c r="S37" t="str">
+        <v/>
+      </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
+      <c r="U37" t="str">
+        <v/>
+      </c>
+      <c r="V37" t="str">
+        <v/>
+      </c>
+      <c r="W37" t="str">
+        <v/>
+      </c>
+      <c r="X37" t="str">
+        <v/>
+      </c>
+      <c r="Y37" t="str">
+        <v/>
+      </c>
+      <c r="Z37" t="str">
+        <v/>
+      </c>
+      <c r="AA37" t="str">
+        <v/>
+      </c>
+      <c r="AB37" t="str">
+        <v/>
+      </c>
+      <c r="AC37" t="str">
+        <v/>
+      </c>
+      <c r="AD37" t="str">
+        <v/>
+      </c>
+      <c r="AE37" t="str">
+        <v/>
+      </c>
+      <c r="AF37" t="str">
+        <v/>
+      </c>
+      <c r="AG37" t="str">
+        <v/>
+      </c>
+      <c r="AH37" t="str">
+        <v/>
+      </c>
+      <c r="AI37">
+        <v>0</v>
+      </c>
+      <c r="AJ37">
+        <v>0</v>
+      </c>
+      <c r="AK37">
+        <v>0</v>
+      </c>
+      <c r="AL37">
+        <v>0</v>
+      </c>
+      <c r="AM37">
+        <v>0</v>
+      </c>
+      <c r="AN37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v/>
+      </c>
+      <c r="B38" t="str">
+        <v>41861</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Phan Hiền Phúc Đạt</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v/>
+      </c>
+      <c r="V38" t="str">
+        <v/>
+      </c>
+      <c r="W38" t="str">
+        <v/>
+      </c>
+      <c r="X38" t="str">
+        <v/>
+      </c>
+      <c r="Y38" t="str">
+        <v/>
+      </c>
+      <c r="Z38" t="str">
+        <v/>
+      </c>
+      <c r="AA38" t="str">
+        <v/>
+      </c>
+      <c r="AB38" t="str">
+        <v/>
+      </c>
+      <c r="AC38" t="str">
+        <v/>
+      </c>
+      <c r="AD38" t="str">
+        <v/>
+      </c>
+      <c r="AE38" t="str">
+        <v/>
+      </c>
+      <c r="AF38" t="str">
+        <v/>
+      </c>
+      <c r="AG38" t="str">
+        <v/>
+      </c>
+      <c r="AH38" t="str">
+        <v/>
+      </c>
+      <c r="AI38">
+        <v>0</v>
+      </c>
+      <c r="AJ38">
+        <v>0</v>
+      </c>
+      <c r="AK38">
+        <v>0</v>
+      </c>
+      <c r="AL38">
+        <v>0</v>
+      </c>
+      <c r="AM38">
+        <v>0</v>
+      </c>
+      <c r="AN38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v/>
+      </c>
+      <c r="B39" t="str">
+        <v>42791</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Nguyễn Phương Linh</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v/>
+      </c>
+      <c r="O39" t="str">
+        <v/>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
+      <c r="R39" t="str">
+        <v/>
+      </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
+      <c r="W39" t="str">
+        <v/>
+      </c>
+      <c r="X39" t="str">
+        <v/>
+      </c>
+      <c r="Y39" t="str">
+        <v/>
+      </c>
+      <c r="Z39" t="str">
+        <v/>
+      </c>
+      <c r="AA39" t="str">
+        <v/>
+      </c>
+      <c r="AB39" t="str">
+        <v/>
+      </c>
+      <c r="AC39" t="str">
+        <v/>
+      </c>
+      <c r="AD39" t="str">
+        <v/>
+      </c>
+      <c r="AE39" t="str">
+        <v/>
+      </c>
+      <c r="AF39" t="str">
+        <v/>
+      </c>
+      <c r="AG39" t="str">
+        <v/>
+      </c>
+      <c r="AH39" t="str">
+        <v/>
+      </c>
+      <c r="AI39">
+        <v>0</v>
+      </c>
+      <c r="AJ39">
+        <v>0</v>
+      </c>
+      <c r="AK39">
+        <v>0</v>
+      </c>
+      <c r="AL39">
+        <v>0</v>
+      </c>
+      <c r="AM39">
+        <v>0</v>
+      </c>
+      <c r="AN39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
+      <c r="B40" t="str">
+        <v>42789</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Nguyễn Phạm Quỳnh Trang</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v/>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+      <c r="N40" t="str">
+        <v/>
+      </c>
+      <c r="O40" t="str">
+        <v/>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v/>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
+      <c r="W40" t="str">
+        <v/>
+      </c>
+      <c r="X40" t="str">
+        <v/>
+      </c>
+      <c r="Y40" t="str">
+        <v/>
+      </c>
+      <c r="Z40" t="str">
+        <v/>
+      </c>
+      <c r="AA40" t="str">
+        <v/>
+      </c>
+      <c r="AB40" t="str">
+        <v/>
+      </c>
+      <c r="AC40" t="str">
+        <v/>
+      </c>
+      <c r="AD40" t="str">
+        <v/>
+      </c>
+      <c r="AE40" t="str">
+        <v/>
+      </c>
+      <c r="AF40" t="str">
+        <v/>
+      </c>
+      <c r="AG40" t="str">
+        <v/>
+      </c>
+      <c r="AH40" t="str">
+        <v/>
+      </c>
+      <c r="AI40">
+        <v>0</v>
+      </c>
+      <c r="AJ40">
+        <v>0</v>
+      </c>
+      <c r="AK40">
+        <v>0</v>
+      </c>
+      <c r="AL40">
+        <v>0</v>
+      </c>
+      <c r="AM40">
+        <v>0</v>
+      </c>
+      <c r="AN40">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>